<commit_message>
Update charts, add Cooling Cost page, restrict to five cities, dashboard improvements
</commit_message>
<xml_diff>
--- a/Final.Project.Data.xlsx
+++ b/Final.Project.Data.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\croni\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://colostate-my.sharepoint.com/personal/c829804536_colostate_edu/Documents/Microsoft Teams Chat Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{143D07AB-F20C-4929-836A-E19FFE3DAE4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="254" documentId="13_ncr:1_{143D07AB-F20C-4929-836A-E19FFE3DAE4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C746725-B97D-4681-AF7A-E0B19B96D811}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{83A2F5A8-6268-4F4A-A0FD-FC6B17854872}"/>
+    <workbookView xWindow="10470" yWindow="0" windowWidth="18330" windowHeight="15585" activeTab="1" xr2:uid="{83A2F5A8-6268-4F4A-A0FD-FC6B17854872}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Cooling Cost Method" sheetId="2" r:id="rId2"/>
+    <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Reduced List" sheetId="3" r:id="rId2"/>
+    <sheet name="Cooling Cost Method" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="78">
   <si>
     <t>city name</t>
   </si>
@@ -237,6 +238,42 @@
     <t>Drift      (gpm)</t>
   </si>
   <si>
+    <t>Peak Makeup (gpm)</t>
+  </si>
+  <si>
+    <t>Peak Makeup (MGD)</t>
+  </si>
+  <si>
+    <t>Peak Annual Makeup (MGY)</t>
+  </si>
+  <si>
+    <t>Actual Annual Makeup (MGY)</t>
+  </si>
+  <si>
+    <t>Data Center Type</t>
+  </si>
+  <si>
+    <t>AI/ML Cluster</t>
+  </si>
+  <si>
+    <t>Hyperscale Cloud</t>
+  </si>
+  <si>
+    <t>Cold and Dry</t>
+  </si>
+  <si>
+    <t>Hot and Wet</t>
+  </si>
+  <si>
+    <t>Hot and Dry</t>
+  </si>
+  <si>
+    <t>Cold and Wet</t>
+  </si>
+  <si>
+    <t>Moderate</t>
+  </si>
+  <si>
     <r>
       <t>Range            (</t>
     </r>
@@ -248,51 +285,38 @@
         <rFont val="Aptos Narrow"/>
         <family val="2"/>
       </rPr>
-      <t>°F)</t>
+      <t>°C)</t>
     </r>
   </si>
   <si>
-    <t>Peak Makeup (gpm)</t>
-  </si>
-  <si>
-    <t>Peak Makeup (MGD)</t>
-  </si>
-  <si>
-    <t>Peak Annual Makeup (MGY)</t>
-  </si>
-  <si>
-    <t>Actual Annual Makeup (MGY)</t>
-  </si>
-  <si>
-    <t>City 2</t>
-  </si>
-  <si>
-    <t>Data Center Type</t>
-  </si>
-  <si>
-    <t>AI/ML Cluster</t>
-  </si>
-  <si>
-    <t>Hyperscale Cloud</t>
-  </si>
-  <si>
-    <t>City 3</t>
-  </si>
-  <si>
-    <t>City 4</t>
-  </si>
-  <si>
-    <t>City 5</t>
+    <t>Electricity Cost ($/kWh)</t>
+  </si>
+  <si>
+    <t>Water Cost ($/1000 gal)</t>
+  </si>
+  <si>
+    <t>Electricity Rate ($/kWh)</t>
+  </si>
+  <si>
+    <t>Water Rate ($/1000 gal)</t>
+  </si>
+  <si>
+    <t>Total Electricity Cost ($/year)</t>
+  </si>
+  <si>
+    <t>Total Water Cost ($/year)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -328,6 +352,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -361,7 +391,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -504,11 +534,189 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -549,6 +757,45 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -578,34 +825,142 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="3" borderId="20" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -629,13 +984,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>114300</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>69850</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>19050</xdr:colOff>
       <xdr:row>39</xdr:row>
       <xdr:rowOff>69850</xdr:rowOff>
@@ -900,10 +1255,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1224,80 +1575,80 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25700A47-9191-47ED-9C7A-28217B165E68}">
   <dimension ref="B3:N34"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.26953125" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.54296875" customWidth="1"/>
-    <col min="6" max="6" width="15.81640625" customWidth="1"/>
-    <col min="7" max="7" width="14.453125" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15.85546875" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
     <col min="8" max="8" width="21" customWidth="1"/>
-    <col min="9" max="9" width="12.26953125" customWidth="1"/>
-    <col min="10" max="10" width="15.7265625" customWidth="1"/>
-    <col min="11" max="11" width="13.54296875" customWidth="1"/>
-    <col min="12" max="12" width="17.453125" customWidth="1"/>
-    <col min="13" max="13" width="18.54296875" customWidth="1"/>
+    <col min="9" max="9" width="12.28515625" customWidth="1"/>
+    <col min="10" max="10" width="15.7109375" customWidth="1"/>
+    <col min="11" max="11" width="13.5703125" customWidth="1"/>
+    <col min="12" max="12" width="17.42578125" customWidth="1"/>
+    <col min="13" max="13" width="18.5703125" customWidth="1"/>
     <col min="14" max="14" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="F4" s="19" t="s">
+    <row r="3" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="F4" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="I4" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="16" t="s">
+      <c r="J4" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="16" t="s">
+      <c r="K4" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="L4" s="16" t="s">
+      <c r="L4" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="M4" s="16" t="s">
+      <c r="M4" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="N4" s="22" t="s">
+      <c r="N4" s="35" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="F5" s="20"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="23"/>
-    </row>
-    <row r="6" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="15" t="s">
+    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="F5" s="33"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="30"/>
+      <c r="L5" s="30"/>
+      <c r="M5" s="30"/>
+      <c r="N5" s="36"/>
+    </row>
+    <row r="6" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
-      <c r="N6" s="24"/>
-    </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
+      <c r="J6" s="31"/>
+      <c r="K6" s="31"/>
+      <c r="L6" s="31"/>
+      <c r="M6" s="31"/>
+      <c r="N6" s="37"/>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>10</v>
       </c>
@@ -1335,7 +1686,7 @@
         <v>0.73330073299999998</v>
       </c>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>13</v>
       </c>
@@ -1373,7 +1724,7 @@
         <v>0.71791360999999998</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B9" s="13" t="s">
         <v>16</v>
       </c>
@@ -1411,7 +1762,7 @@
         <v>0.45251833699999999</v>
       </c>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>18</v>
       </c>
@@ -1449,7 +1800,7 @@
         <v>0.75693561499999995</v>
       </c>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B11" s="14" t="s">
         <v>21</v>
       </c>
@@ -1487,7 +1838,7 @@
         <v>0.51339853300000005</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>24</v>
       </c>
@@ -1525,7 +1876,7 @@
         <v>0.82</v>
       </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
       <c r="F13" s="8" t="s">
         <v>27</v>
       </c>
@@ -1554,7 +1905,7 @@
         <v>0.82</v>
       </c>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
       <c r="F14" s="6" t="s">
         <v>28</v>
       </c>
@@ -1583,7 +1934,7 @@
         <v>0.73861450699999998</v>
       </c>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>29</v>
       </c>
@@ -1615,7 +1966,7 @@
         <v>0.68513447400000005</v>
       </c>
     </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>31</v>
       </c>
@@ -1647,7 +1998,7 @@
         <v>0.73861450699999998</v>
       </c>
     </row>
-    <row r="17" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="17" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F17" s="8" t="s">
         <v>33</v>
       </c>
@@ -1676,7 +2027,7 @@
         <v>0.73861450699999998</v>
       </c>
     </row>
-    <row r="18" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="18" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F18" s="6" t="s">
         <v>34</v>
       </c>
@@ -1705,7 +2056,7 @@
         <v>0.63240423800000001</v>
       </c>
     </row>
-    <row r="19" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="19" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F19" s="8" t="s">
         <v>35</v>
       </c>
@@ -1734,7 +2085,7 @@
         <v>0.84718826400000002</v>
       </c>
     </row>
-    <row r="20" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="20" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F20" s="6" t="s">
         <v>36</v>
       </c>
@@ -1763,7 +2114,7 @@
         <v>0.63240423800000001</v>
       </c>
     </row>
-    <row r="21" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="21" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F21" s="8" t="s">
         <v>37</v>
       </c>
@@ -1792,7 +2143,7 @@
         <v>0.65204563999999998</v>
       </c>
     </row>
-    <row r="22" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="22" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F22" s="6" t="s">
         <v>38</v>
       </c>
@@ -1821,7 +2172,7 @@
         <v>0.61828850899999999</v>
       </c>
     </row>
-    <row r="23" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="23" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F23" s="8" t="s">
         <v>39</v>
       </c>
@@ -1850,7 +2201,7 @@
         <v>0.75693561499999995</v>
       </c>
     </row>
-    <row r="24" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="24" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F24" s="6" t="s">
         <v>40</v>
       </c>
@@ -1879,7 +2230,7 @@
         <v>0.46995925</v>
       </c>
     </row>
-    <row r="25" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="25" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F25" s="8" t="s">
         <v>41</v>
       </c>
@@ -1908,7 +2259,7 @@
         <v>0.65204563999999998</v>
       </c>
     </row>
-    <row r="26" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="26" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F26" s="6" t="s">
         <v>42</v>
       </c>
@@ -1937,7 +2288,7 @@
         <v>0.84718826400000002</v>
       </c>
     </row>
-    <row r="27" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="27" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F27" s="8" t="s">
         <v>43</v>
       </c>
@@ -1966,7 +2317,7 @@
         <v>0.82</v>
       </c>
     </row>
-    <row r="28" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="28" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F28" s="6" t="s">
         <v>44</v>
       </c>
@@ -1995,7 +2346,7 @@
         <v>0.13457212700000001</v>
       </c>
     </row>
-    <row r="29" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="29" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F29" s="8" t="s">
         <v>45</v>
       </c>
@@ -2024,7 +2375,7 @@
         <v>0.73861450699999998</v>
       </c>
     </row>
-    <row r="30" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="30" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F30" s="6" t="s">
         <v>46</v>
       </c>
@@ -2053,7 +2404,7 @@
         <v>0.61268133700000005</v>
       </c>
     </row>
-    <row r="31" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="31" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F31" s="8" t="s">
         <v>47</v>
       </c>
@@ -2082,7 +2433,7 @@
         <v>0.59303993499999996</v>
       </c>
     </row>
-    <row r="32" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="32" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F32" s="6" t="s">
         <v>48</v>
       </c>
@@ -2111,7 +2462,7 @@
         <v>0.13457212700000001</v>
       </c>
     </row>
-    <row r="33" spans="6:14" x14ac:dyDescent="0.35">
+    <row r="33" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F33" s="8" t="s">
         <v>49</v>
       </c>
@@ -2140,7 +2491,7 @@
         <v>0.85343113299999995</v>
       </c>
     </row>
-    <row r="34" spans="6:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="6:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F34" s="10" t="s">
         <v>50</v>
       </c>
@@ -2190,554 +2541,1760 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD78BB6E-C1C0-4A9D-BA3C-923E087DD123}">
-  <dimension ref="A1:N11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67D9E650-CBDC-48FD-9FE1-D900660452A4}">
+  <dimension ref="C6:P37"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.6328125" style="26" customWidth="1"/>
-    <col min="2" max="2" width="15.6328125" style="26" customWidth="1"/>
-    <col min="3" max="3" width="10.6328125" style="26" customWidth="1"/>
-    <col min="4" max="4" width="10.6328125" style="29" customWidth="1"/>
-    <col min="5" max="6" width="10.6328125" style="26" customWidth="1"/>
-    <col min="7" max="7" width="10.6328125" style="33" customWidth="1"/>
-    <col min="8" max="13" width="10.6328125" style="26" customWidth="1"/>
+    <col min="5" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" customWidth="1"/>
+    <col min="9" max="9" width="13.42578125" customWidth="1"/>
+    <col min="10" max="10" width="15" customWidth="1"/>
+    <col min="11" max="11" width="12.28515625" customWidth="1"/>
+    <col min="12" max="13" width="14" customWidth="1"/>
+    <col min="14" max="14" width="11" customWidth="1"/>
+    <col min="15" max="15" width="13.85546875" customWidth="1"/>
+    <col min="16" max="16" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="25" customFormat="1" ht="58" x14ac:dyDescent="0.35">
-      <c r="A1" s="27" t="s">
+    <row r="6" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="E7" s="32" t="s">
+        <v>0</v>
+      </c>
+      <c r="F7" s="44" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" s="44" t="s">
+        <v>73</v>
+      </c>
+      <c r="H7" s="29" t="s">
+        <v>1</v>
+      </c>
+      <c r="I7" s="29" t="s">
+        <v>2</v>
+      </c>
+      <c r="J7" s="29" t="s">
+        <v>3</v>
+      </c>
+      <c r="K7" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="L7" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="M7" s="29" t="s">
+        <v>6</v>
+      </c>
+      <c r="N7" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="O7" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="P7" s="51"/>
+    </row>
+    <row r="8" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="E8" s="33"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="45"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30"/>
+      <c r="K8" s="30"/>
+      <c r="L8" s="30"/>
+      <c r="M8" s="30"/>
+      <c r="N8" s="30"/>
+      <c r="O8" s="36"/>
+      <c r="P8" s="51"/>
+    </row>
+    <row r="9" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E9" s="34"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="31"/>
+      <c r="J9" s="31"/>
+      <c r="K9" s="31"/>
+      <c r="L9" s="31"/>
+      <c r="M9" s="31"/>
+      <c r="N9" s="31"/>
+      <c r="O9" s="37"/>
+      <c r="P9" s="51"/>
+    </row>
+    <row r="10" spans="5:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="40"/>
+      <c r="G10" s="40"/>
+      <c r="H10" s="4">
+        <v>16.033999999999999</v>
+      </c>
+      <c r="I10" s="4">
+        <v>108.383</v>
+      </c>
+      <c r="J10" s="4">
+        <v>0.499</v>
+      </c>
+      <c r="K10" s="4">
+        <v>13604</v>
+      </c>
+      <c r="L10" s="4">
+        <v>6789</v>
+      </c>
+      <c r="M10" s="4">
+        <v>906660</v>
+      </c>
+      <c r="N10" s="4">
+        <v>3</v>
+      </c>
+      <c r="O10" s="5">
+        <v>0.73330073299999998</v>
+      </c>
+    </row>
+    <row r="11" spans="5:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="41"/>
+      <c r="G11" s="41"/>
+      <c r="H11" s="2">
+        <v>19.849</v>
+      </c>
+      <c r="I11" s="2">
+        <v>70.185000000000002</v>
+      </c>
+      <c r="J11" s="2">
+        <v>0.43099999999999999</v>
+      </c>
+      <c r="K11" s="2">
+        <v>13604</v>
+      </c>
+      <c r="L11" s="2">
+        <v>5864</v>
+      </c>
+      <c r="M11" s="2">
+        <v>906660</v>
+      </c>
+      <c r="N11" s="2">
+        <v>4</v>
+      </c>
+      <c r="O11" s="7">
+        <v>0.71791360999999998</v>
+      </c>
+    </row>
+    <row r="12" spans="5:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E12" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" s="42"/>
+      <c r="G12" s="42"/>
+      <c r="H12" s="1">
+        <v>9.5210000000000008</v>
+      </c>
+      <c r="I12" s="1">
+        <v>95.132999999999996</v>
+      </c>
+      <c r="J12" s="1">
+        <v>0.36299999999999999</v>
+      </c>
+      <c r="K12" s="1">
+        <v>11238</v>
+      </c>
+      <c r="L12" s="1">
+        <v>4080</v>
+      </c>
+      <c r="M12" s="1">
+        <v>748980</v>
+      </c>
+      <c r="N12" s="1">
+        <v>2</v>
+      </c>
+      <c r="O12" s="9">
+        <v>0.45251833699999999</v>
+      </c>
+    </row>
+    <row r="13" spans="5:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E13" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" s="41"/>
+      <c r="G13" s="41"/>
+      <c r="H13" s="2">
+        <v>15.423999999999999</v>
+      </c>
+      <c r="I13" s="2">
+        <v>96.49</v>
+      </c>
+      <c r="J13" s="2">
+        <v>0.54400000000000004</v>
+      </c>
+      <c r="K13" s="2">
+        <v>13013</v>
+      </c>
+      <c r="L13" s="2">
+        <v>7079</v>
+      </c>
+      <c r="M13" s="2">
+        <v>867240</v>
+      </c>
+      <c r="N13" s="2">
+        <v>3</v>
+      </c>
+      <c r="O13" s="7">
+        <v>0.75693561499999995</v>
+      </c>
+    </row>
+    <row r="14" spans="5:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E14" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" s="42"/>
+      <c r="G14" s="42"/>
+      <c r="H14" s="1">
+        <v>9.8810000000000002</v>
+      </c>
+      <c r="I14" s="1">
+        <v>73.608999999999995</v>
+      </c>
+      <c r="J14" s="1">
+        <v>0.40799999999999997</v>
+      </c>
+      <c r="K14" s="1">
+        <v>11830</v>
+      </c>
+      <c r="L14" s="1">
+        <v>4827</v>
+      </c>
+      <c r="M14" s="1">
+        <v>788400</v>
+      </c>
+      <c r="N14" s="1">
+        <v>2</v>
+      </c>
+      <c r="O14" s="9">
+        <v>0.51339853300000005</v>
+      </c>
+    </row>
+    <row r="15" spans="5:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E15" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" s="41"/>
+      <c r="G15" s="41"/>
+      <c r="H15" s="2">
+        <v>10.324</v>
+      </c>
+      <c r="I15" s="2">
+        <v>74.114999999999995</v>
+      </c>
+      <c r="J15" s="2">
+        <v>0.72599999999999998</v>
+      </c>
+      <c r="K15" s="2">
+        <v>11830</v>
+      </c>
+      <c r="L15" s="2">
+        <v>8589</v>
+      </c>
+      <c r="M15" s="2">
+        <v>788400</v>
+      </c>
+      <c r="N15" s="2">
+        <v>2</v>
+      </c>
+      <c r="O15" s="7">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="16" spans="5:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E16" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="42"/>
+      <c r="G16" s="42"/>
+      <c r="H16" s="1">
+        <v>11.242000000000001</v>
+      </c>
+      <c r="I16" s="1">
+        <v>82.866</v>
+      </c>
+      <c r="J16" s="1">
+        <v>0.72599999999999998</v>
+      </c>
+      <c r="K16" s="1">
+        <v>11830</v>
+      </c>
+      <c r="L16" s="1">
+        <v>8589</v>
+      </c>
+      <c r="M16" s="1">
+        <v>788400</v>
+      </c>
+      <c r="N16" s="1">
+        <v>2</v>
+      </c>
+      <c r="O16" s="9">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="17" spans="3:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E17" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="41"/>
+      <c r="G17" s="41"/>
+      <c r="H17" s="2">
+        <v>18.763999999999999</v>
+      </c>
+      <c r="I17" s="2">
+        <v>76.909000000000006</v>
+      </c>
+      <c r="J17" s="2">
+        <v>0.43099999999999999</v>
+      </c>
+      <c r="K17" s="2">
+        <v>14196</v>
+      </c>
+      <c r="L17" s="2">
+        <v>6118</v>
+      </c>
+      <c r="M17" s="2">
+        <v>946080</v>
+      </c>
+      <c r="N17" s="2">
+        <v>4</v>
+      </c>
+      <c r="O17" s="7">
+        <v>0.73861450699999998</v>
+      </c>
+    </row>
+    <row r="18" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C18" s="28" t="s">
+        <v>66</v>
+      </c>
+      <c r="D18" s="38"/>
+      <c r="E18" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" s="47">
+        <v>0.13300000000000001</v>
+      </c>
+      <c r="G18" s="47">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="H18" s="2">
+        <v>10.233000000000001</v>
+      </c>
+      <c r="I18" s="2">
+        <v>30.747</v>
+      </c>
+      <c r="J18" s="2">
+        <v>0.499</v>
+      </c>
+      <c r="K18" s="2">
+        <v>12422</v>
+      </c>
+      <c r="L18" s="2">
+        <v>6198</v>
+      </c>
+      <c r="M18" s="2">
+        <v>827820</v>
+      </c>
+      <c r="N18" s="2">
+        <v>3</v>
+      </c>
+      <c r="O18" s="7">
+        <v>0.68513447400000005</v>
+      </c>
+    </row>
+    <row r="19" spans="3:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E19" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F19" s="47"/>
+      <c r="G19" s="47"/>
+      <c r="H19" s="2">
+        <v>18.771999999999998</v>
+      </c>
+      <c r="I19" s="2">
+        <v>70.992000000000004</v>
+      </c>
+      <c r="J19" s="2">
+        <v>0.43099999999999999</v>
+      </c>
+      <c r="K19" s="2">
+        <v>14196</v>
+      </c>
+      <c r="L19" s="2">
+        <v>6118</v>
+      </c>
+      <c r="M19" s="2">
+        <v>946080</v>
+      </c>
+      <c r="N19" s="2">
+        <v>4</v>
+      </c>
+      <c r="O19" s="7">
+        <v>0.73861450699999998</v>
+      </c>
+    </row>
+    <row r="20" spans="3:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E20" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F20" s="48"/>
+      <c r="G20" s="48"/>
+      <c r="H20" s="1">
+        <v>20.689</v>
+      </c>
+      <c r="I20" s="1">
+        <v>101.946</v>
+      </c>
+      <c r="J20" s="1">
+        <v>0.43099999999999999</v>
+      </c>
+      <c r="K20" s="1">
+        <v>14196</v>
+      </c>
+      <c r="L20" s="1">
+        <v>6118</v>
+      </c>
+      <c r="M20" s="1">
+        <v>946080</v>
+      </c>
+      <c r="N20" s="1">
+        <v>4</v>
+      </c>
+      <c r="O20" s="9">
+        <v>0.73861450699999998</v>
+      </c>
+    </row>
+    <row r="21" spans="3:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E21" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F21" s="47"/>
+      <c r="G21" s="47"/>
+      <c r="H21" s="2">
+        <v>20.268000000000001</v>
+      </c>
+      <c r="I21" s="2">
+        <v>105.20099999999999</v>
+      </c>
+      <c r="J21" s="2">
+        <v>0.40799999999999997</v>
+      </c>
+      <c r="K21" s="2">
+        <v>13604</v>
+      </c>
+      <c r="L21" s="2">
+        <v>5551</v>
+      </c>
+      <c r="M21" s="2">
+        <v>906660</v>
+      </c>
+      <c r="N21" s="2">
+        <v>3</v>
+      </c>
+      <c r="O21" s="7">
+        <v>0.63240423800000001</v>
+      </c>
+    </row>
+    <row r="22" spans="3:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E22" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F22" s="48"/>
+      <c r="G22" s="48"/>
+      <c r="H22" s="1">
+        <v>19.584</v>
+      </c>
+      <c r="I22" s="1">
+        <v>9.14</v>
+      </c>
+      <c r="J22" s="1">
+        <v>0.45400000000000001</v>
+      </c>
+      <c r="K22" s="1">
+        <v>14788</v>
+      </c>
+      <c r="L22" s="1">
+        <v>6714</v>
+      </c>
+      <c r="M22" s="1">
+        <v>985500</v>
+      </c>
+      <c r="N22" s="1">
+        <v>5</v>
+      </c>
+      <c r="O22" s="9">
+        <v>0.84718826400000002</v>
+      </c>
+    </row>
+    <row r="23" spans="3:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E23" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F23" s="47"/>
+      <c r="G23" s="47"/>
+      <c r="H23" s="2">
+        <v>17.655000000000001</v>
+      </c>
+      <c r="I23" s="2">
+        <v>31.876999999999999</v>
+      </c>
+      <c r="J23" s="2">
+        <v>0.40799999999999997</v>
+      </c>
+      <c r="K23" s="2">
+        <v>13604</v>
+      </c>
+      <c r="L23" s="2">
+        <v>5551</v>
+      </c>
+      <c r="M23" s="2">
+        <v>906660</v>
+      </c>
+      <c r="N23" s="2">
+        <v>3</v>
+      </c>
+      <c r="O23" s="7">
+        <v>0.63240423800000001</v>
+      </c>
+    </row>
+    <row r="24" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C24" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="D24" s="38"/>
+      <c r="E24" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F24" s="48">
+        <v>0.11600000000000001</v>
+      </c>
+      <c r="G24" s="48">
+        <v>5.5</v>
+      </c>
+      <c r="H24" s="1">
+        <v>24.181000000000001</v>
+      </c>
+      <c r="I24" s="1">
+        <v>120.622</v>
+      </c>
+      <c r="J24" s="1">
+        <v>0.40799999999999997</v>
+      </c>
+      <c r="K24" s="1">
+        <v>14196</v>
+      </c>
+      <c r="L24" s="1">
+        <v>5792</v>
+      </c>
+      <c r="M24" s="1">
+        <v>946080</v>
+      </c>
+      <c r="N24" s="1">
+        <v>3</v>
+      </c>
+      <c r="O24" s="9">
+        <v>0.65204563999999998</v>
+      </c>
+    </row>
+    <row r="25" spans="3:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="D25" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F25" s="47"/>
+      <c r="G25" s="47"/>
+      <c r="H25" s="2">
+        <v>6.87</v>
+      </c>
+      <c r="I25" s="2">
+        <v>62.133000000000003</v>
+      </c>
+      <c r="J25" s="2">
+        <v>0.54400000000000004</v>
+      </c>
+      <c r="K25" s="2">
+        <v>11238</v>
+      </c>
+      <c r="L25" s="2">
+        <v>6114</v>
+      </c>
+      <c r="M25" s="2">
+        <v>748980</v>
+      </c>
+      <c r="N25" s="2">
+        <v>2</v>
+      </c>
+      <c r="O25" s="7">
+        <v>0.61828850899999999</v>
+      </c>
+    </row>
+    <row r="26" spans="3:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E26" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F26" s="48"/>
+      <c r="G26" s="48"/>
+      <c r="H26" s="1">
+        <v>14.941000000000001</v>
+      </c>
+      <c r="I26" s="1">
+        <v>102.905</v>
+      </c>
+      <c r="J26" s="1">
+        <v>0.54400000000000004</v>
+      </c>
+      <c r="K26" s="1">
+        <v>13013</v>
+      </c>
+      <c r="L26" s="1">
+        <v>7079</v>
+      </c>
+      <c r="M26" s="1">
+        <v>867240</v>
+      </c>
+      <c r="N26" s="1">
+        <v>3</v>
+      </c>
+      <c r="O26" s="9">
+        <v>0.75693561499999995</v>
+      </c>
+    </row>
+    <row r="27" spans="3:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E27" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F27" s="47"/>
+      <c r="G27" s="47"/>
+      <c r="H27" s="2">
+        <v>11.968999999999999</v>
+      </c>
+      <c r="I27" s="2">
+        <v>96.614000000000004</v>
+      </c>
+      <c r="J27" s="2">
+        <v>0.36299999999999999</v>
+      </c>
+      <c r="K27" s="2">
+        <v>11830</v>
+      </c>
+      <c r="L27" s="2">
+        <v>4294</v>
+      </c>
+      <c r="M27" s="2">
+        <v>788400</v>
+      </c>
+      <c r="N27" s="2">
+        <v>2</v>
+      </c>
+      <c r="O27" s="7">
+        <v>0.46995925</v>
+      </c>
+    </row>
+    <row r="28" spans="3:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E28" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="F28" s="48"/>
+      <c r="G28" s="48"/>
+      <c r="H28" s="1">
+        <v>22.093</v>
+      </c>
+      <c r="I28" s="1">
+        <v>107.021</v>
+      </c>
+      <c r="J28" s="1">
+        <v>0.40799999999999997</v>
+      </c>
+      <c r="K28" s="1">
+        <v>14196</v>
+      </c>
+      <c r="L28" s="1">
+        <v>5792</v>
+      </c>
+      <c r="M28" s="1">
+        <v>946080</v>
+      </c>
+      <c r="N28" s="1">
+        <v>3</v>
+      </c>
+      <c r="O28" s="9">
+        <v>0.65204563999999998</v>
+      </c>
+    </row>
+    <row r="29" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C29" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="D29" s="38"/>
+      <c r="E29" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F29" s="47">
+        <v>0.13100000000000001</v>
+      </c>
+      <c r="G29" s="47">
+        <v>3.5</v>
+      </c>
+      <c r="H29" s="2">
+        <v>21.507999999999999</v>
+      </c>
+      <c r="I29" s="2">
+        <v>16.231000000000002</v>
+      </c>
+      <c r="J29" s="2">
+        <v>0.45400000000000001</v>
+      </c>
+      <c r="K29" s="2">
+        <v>14788</v>
+      </c>
+      <c r="L29" s="2">
+        <v>6714</v>
+      </c>
+      <c r="M29" s="2">
+        <v>985500</v>
+      </c>
+      <c r="N29" s="2">
+        <v>5</v>
+      </c>
+      <c r="O29" s="7">
+        <v>0.84718826400000002</v>
+      </c>
+    </row>
+    <row r="30" spans="3:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E30" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F30" s="48"/>
+      <c r="G30" s="48"/>
+      <c r="H30" s="1">
+        <v>11.009</v>
+      </c>
+      <c r="I30" s="1">
+        <v>80.269000000000005</v>
+      </c>
+      <c r="J30" s="1">
+        <v>0.72599999999999998</v>
+      </c>
+      <c r="K30" s="1">
+        <v>11830</v>
+      </c>
+      <c r="L30" s="1">
+        <v>8589</v>
+      </c>
+      <c r="M30" s="1">
+        <v>788400</v>
+      </c>
+      <c r="N30" s="1">
+        <v>2</v>
+      </c>
+      <c r="O30" s="9">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="31" spans="3:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E31" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F31" s="47"/>
+      <c r="G31" s="47"/>
+      <c r="H31" s="2">
+        <v>11.555999999999999</v>
+      </c>
+      <c r="I31" s="2">
+        <v>82.534999999999997</v>
+      </c>
+      <c r="J31" s="2">
+        <v>9.0999999999999998E-2</v>
+      </c>
+      <c r="K31" s="2">
+        <v>10056</v>
+      </c>
+      <c r="L31" s="2">
+        <v>915</v>
+      </c>
+      <c r="M31" s="2">
+        <v>670140</v>
+      </c>
+      <c r="N31" s="2">
+        <v>1</v>
+      </c>
+      <c r="O31" s="7">
+        <v>0.13457212700000001</v>
+      </c>
+    </row>
+    <row r="32" spans="3:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E32" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="F32" s="48"/>
+      <c r="G32" s="48"/>
+      <c r="H32" s="1">
+        <v>20.606999999999999</v>
+      </c>
+      <c r="I32" s="1">
+        <v>62.13</v>
+      </c>
+      <c r="J32" s="1">
+        <v>0.43099999999999999</v>
+      </c>
+      <c r="K32" s="1">
+        <v>14196</v>
+      </c>
+      <c r="L32" s="1">
+        <v>6118</v>
+      </c>
+      <c r="M32" s="1">
+        <v>946080</v>
+      </c>
+      <c r="N32" s="1">
+        <v>4</v>
+      </c>
+      <c r="O32" s="9">
+        <v>0.73861450699999998</v>
+      </c>
+    </row>
+    <row r="33" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C33" s="28" t="s">
+        <v>70</v>
+      </c>
+      <c r="D33" s="38"/>
+      <c r="E33" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="F33" s="48">
+        <v>0.29499999999999998</v>
+      </c>
+      <c r="G33" s="48">
+        <v>11.5</v>
+      </c>
+      <c r="H33" s="1">
+        <v>16.437999999999999</v>
+      </c>
+      <c r="I33" s="1">
+        <v>21.013999999999999</v>
+      </c>
+      <c r="J33" s="1">
+        <v>0.40799999999999997</v>
+      </c>
+      <c r="K33" s="1">
+        <v>13013</v>
+      </c>
+      <c r="L33" s="1">
+        <v>5309</v>
+      </c>
+      <c r="M33" s="1">
+        <v>867240</v>
+      </c>
+      <c r="N33" s="1">
+        <v>3</v>
+      </c>
+      <c r="O33" s="9">
+        <v>0.61268133700000005</v>
+      </c>
+    </row>
+    <row r="34" spans="3:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E34" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F34" s="48"/>
+      <c r="G34" s="48"/>
+      <c r="H34" s="1">
+        <v>14.919</v>
+      </c>
+      <c r="I34" s="1">
+        <v>30.617999999999999</v>
+      </c>
+      <c r="J34" s="1">
+        <v>0.40799999999999997</v>
+      </c>
+      <c r="K34" s="1">
+        <v>12422</v>
+      </c>
+      <c r="L34" s="1">
+        <v>5068</v>
+      </c>
+      <c r="M34" s="1">
+        <v>827820</v>
+      </c>
+      <c r="N34" s="1">
+        <v>3</v>
+      </c>
+      <c r="O34" s="9">
+        <v>0.59303993499999996</v>
+      </c>
+    </row>
+    <row r="35" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C35" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="D35" s="38"/>
+      <c r="E35" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F35" s="47">
+        <v>0.11899999999999999</v>
+      </c>
+      <c r="G35" s="47">
+        <v>5.5</v>
+      </c>
+      <c r="H35" s="2">
+        <v>11.103</v>
+      </c>
+      <c r="I35" s="2">
+        <v>76.224000000000004</v>
+      </c>
+      <c r="J35" s="2">
+        <v>9.0999999999999998E-2</v>
+      </c>
+      <c r="K35" s="2">
+        <v>10056</v>
+      </c>
+      <c r="L35" s="2">
+        <v>915</v>
+      </c>
+      <c r="M35" s="2">
+        <v>670140</v>
+      </c>
+      <c r="N35" s="2">
+        <v>1</v>
+      </c>
+      <c r="O35" s="7">
+        <v>0.13457212700000001</v>
+      </c>
+    </row>
+    <row r="36" spans="3:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E36" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="F36" s="42"/>
+      <c r="G36" s="42"/>
+      <c r="H36" s="1">
+        <v>13.269</v>
+      </c>
+      <c r="I36" s="1">
+        <v>81.724999999999994</v>
+      </c>
+      <c r="J36" s="1">
+        <v>0.63500000000000001</v>
+      </c>
+      <c r="K36" s="1">
+        <v>13013</v>
+      </c>
+      <c r="L36" s="1">
+        <v>8263</v>
+      </c>
+      <c r="M36" s="1">
+        <v>867240</v>
+      </c>
+      <c r="N36" s="1">
+        <v>3</v>
+      </c>
+      <c r="O36" s="9">
+        <v>0.85343113299999995</v>
+      </c>
+    </row>
+    <row r="37" spans="3:15" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E37" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="F37" s="43"/>
+      <c r="G37" s="43"/>
+      <c r="H37" s="11">
+        <v>22.565000000000001</v>
+      </c>
+      <c r="I37" s="11">
+        <v>110.053</v>
+      </c>
+      <c r="J37" s="11">
+        <v>0.40799999999999997</v>
+      </c>
+      <c r="K37" s="11">
+        <v>14196</v>
+      </c>
+      <c r="L37" s="11">
+        <v>5792</v>
+      </c>
+      <c r="M37" s="11">
+        <v>946080</v>
+      </c>
+      <c r="N37" s="11">
+        <v>3</v>
+      </c>
+      <c r="O37" s="12">
+        <v>0.65204563999999998</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="17">
+    <mergeCell ref="P7:P9"/>
+    <mergeCell ref="M7:M9"/>
+    <mergeCell ref="N7:N9"/>
+    <mergeCell ref="O7:O9"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="H7:H9"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="J7:J9"/>
+    <mergeCell ref="K7:K9"/>
+    <mergeCell ref="L7:L9"/>
+    <mergeCell ref="G7:G9"/>
+    <mergeCell ref="F7:F9"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD78BB6E-C1C0-4A9D-BA3C-923E087DD123}">
+  <dimension ref="A1:S11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.42578125" customWidth="1"/>
+    <col min="2" max="2" width="20.5703125" style="16" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" style="16" customWidth="1"/>
+    <col min="4" max="5" width="10.5703125" style="16" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" style="16" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" style="17" customWidth="1"/>
+    <col min="8" max="9" width="10.5703125" style="16" customWidth="1"/>
+    <col min="10" max="10" width="10.5703125" style="18" customWidth="1"/>
+    <col min="11" max="16" width="10.5703125" style="16" customWidth="1"/>
+    <col min="18" max="18" width="9.5703125" customWidth="1"/>
+    <col min="19" max="19" width="16.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" s="15" customFormat="1" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="69" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="70" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="70" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="E1" s="76" t="s">
+        <v>74</v>
+      </c>
+      <c r="F1" s="76" t="s">
+        <v>76</v>
+      </c>
+      <c r="G1" s="71" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="27" t="s">
+      <c r="H1" s="70" t="s">
+        <v>71</v>
+      </c>
+      <c r="I1" s="70" t="s">
+        <v>54</v>
+      </c>
+      <c r="J1" s="72" t="s">
+        <v>55</v>
+      </c>
+      <c r="K1" s="70" t="s">
+        <v>57</v>
+      </c>
+      <c r="L1" s="70" t="s">
+        <v>56</v>
+      </c>
+      <c r="M1" s="70" t="s">
+        <v>58</v>
+      </c>
+      <c r="N1" s="70" t="s">
         <v>59</v>
       </c>
-      <c r="F1" s="27" t="s">
-        <v>54</v>
-      </c>
-      <c r="G1" s="32" t="s">
-        <v>55</v>
-      </c>
-      <c r="H1" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="I1" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="J1" s="27" t="s">
-        <v>58</v>
-      </c>
-      <c r="K1" s="27" t="s">
+      <c r="O1" s="70" t="s">
         <v>60</v>
       </c>
-      <c r="L1" s="27" t="s">
+      <c r="P1" s="70" t="s">
         <v>61</v>
       </c>
-      <c r="M1" s="27" t="s">
+      <c r="Q1" s="70" t="s">
         <v>62</v>
       </c>
-      <c r="N1" s="27" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
+      <c r="R1" s="76" t="s">
+        <v>75</v>
+      </c>
+      <c r="S1" s="77" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A2" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="C2" s="26">
+      <c r="C2" s="52" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="52">
         <v>100</v>
       </c>
-      <c r="D2" s="29">
+      <c r="E2" s="53">
+        <v>0.13</v>
+      </c>
+      <c r="F2" s="80">
+        <f>D2*1000*365*E2</f>
+        <v>4745000</v>
+      </c>
+      <c r="G2" s="61">
         <v>0.8</v>
       </c>
-      <c r="E2" s="26">
+      <c r="H2" s="52">
         <f>70-55</f>
         <v>15</v>
       </c>
-      <c r="F2" s="26">
+      <c r="I2" s="52">
         <v>4</v>
       </c>
-      <c r="G2" s="33">
-        <f>C2*1000/3.517</f>
+      <c r="J2" s="62">
+        <f>D2*1000/3.517</f>
         <v>28433.323855558716</v>
       </c>
-      <c r="H2" s="31">
-        <f>0.001*G2*E2</f>
+      <c r="K2" s="63">
+        <f>0.001*J2*H2</f>
         <v>426.4998578333807</v>
       </c>
-      <c r="I2" s="31">
-        <f>H2/(F2-1)</f>
+      <c r="L2" s="63">
+        <f>K2/(I2-1)</f>
         <v>142.16661927779356</v>
       </c>
-      <c r="J2" s="31">
-        <f>0.01*H2</f>
+      <c r="M2" s="63">
+        <f>0.01*K2</f>
         <v>4.2649985783338069</v>
       </c>
-      <c r="K2" s="31">
-        <f>SUM(H2:J2)</f>
+      <c r="N2" s="63">
+        <f>SUM(K2:M2)</f>
         <v>572.93147568950803</v>
       </c>
-      <c r="L2" s="30">
-        <f>K2*60*24/10^6</f>
+      <c r="O2" s="64">
+        <f>N2*60*24/10^6</f>
         <v>0.8250213249928916</v>
       </c>
-      <c r="M2" s="31">
-        <f>L2*365</f>
+      <c r="P2" s="63">
+        <f>O2*365</f>
         <v>301.13278362240544</v>
       </c>
-      <c r="N2" s="31">
-        <f>M2*D2</f>
+      <c r="Q2" s="68">
+        <f>P2*G2</f>
         <v>240.90622689792437</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A3" s="26" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="C3" s="26">
+      <c r="R2" s="53">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="S2" s="78">
+        <f>(Q2*(10^3))*$R$2</f>
+        <v>1180440.5117998295</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="39"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" s="2">
         <v>100</v>
       </c>
-      <c r="D3" s="29">
+      <c r="E3" s="65"/>
+      <c r="F3" s="81"/>
+      <c r="G3" s="20">
         <v>0.6</v>
       </c>
-      <c r="E3" s="26">
+      <c r="H3" s="2">
         <f>70-55</f>
         <v>15</v>
       </c>
-      <c r="F3" s="26">
+      <c r="I3" s="2">
         <v>4</v>
       </c>
-      <c r="G3" s="33">
-        <f>C3*1000/3.517</f>
+      <c r="J3" s="21">
+        <f>D3*1000/3.517</f>
         <v>28433.323855558716</v>
       </c>
-      <c r="H3" s="31">
-        <f>0.001*G3*E3</f>
+      <c r="K3" s="22">
+        <f>0.001*J3*H3</f>
         <v>426.4998578333807</v>
       </c>
-      <c r="I3" s="31">
-        <f>H3/(F3-1)</f>
+      <c r="L3" s="22">
+        <f>K3/(I3-1)</f>
         <v>142.16661927779356</v>
       </c>
-      <c r="J3" s="31">
-        <f>0.01*H3</f>
+      <c r="M3" s="22">
+        <f>0.01*K3</f>
         <v>4.2649985783338069</v>
       </c>
-      <c r="K3" s="31">
-        <f>SUM(H3:J3)</f>
+      <c r="N3" s="22">
+        <f>SUM(K3:M3)</f>
         <v>572.93147568950803</v>
       </c>
-      <c r="L3" s="30">
-        <f>K3*60*24/10^6</f>
+      <c r="O3" s="23">
+        <f>N3*60*24/10^6</f>
         <v>0.8250213249928916</v>
       </c>
-      <c r="M3" s="31">
-        <f>L3*365</f>
+      <c r="P3" s="22">
+        <f>O3*365</f>
         <v>301.13278362240544</v>
       </c>
-      <c r="N3" s="31">
-        <f>M3*D3</f>
+      <c r="Q3" s="66">
+        <f>P3*G3</f>
         <v>180.67967017344327</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A4" s="26" t="s">
+      <c r="R3" s="65"/>
+      <c r="S3" s="78">
+        <f t="shared" ref="S3:S11" si="0">(Q3*(10^3))*$R$2</f>
+        <v>885330.38384987204</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="39" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" s="55" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B4" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="C4" s="26">
+      <c r="D4" s="1">
         <v>100</v>
       </c>
-      <c r="D4" s="29">
+      <c r="E4" s="67">
+        <v>0.12</v>
+      </c>
+      <c r="F4" s="82">
+        <f t="shared" ref="F4" si="1">D4*1000*365*E4</f>
+        <v>4380000</v>
+      </c>
+      <c r="G4" s="57">
         <v>0.8</v>
       </c>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="33">
-        <f t="shared" ref="G4:G11" si="0">C4*1000/3.517</f>
+      <c r="H4" s="1">
+        <v>20</v>
+      </c>
+      <c r="I4" s="1">
+        <v>3</v>
+      </c>
+      <c r="J4" s="58">
+        <f t="shared" ref="J4:J11" si="2">D4*1000/3.517</f>
         <v>28433.323855558716</v>
       </c>
-      <c r="H4" s="31">
-        <f t="shared" ref="H4:H11" si="1">0.001*G4*E4</f>
-        <v>0</v>
-      </c>
-      <c r="I4" s="31">
-        <f t="shared" ref="I4:I11" si="2">H4/(F4-1)</f>
-        <v>0</v>
-      </c>
-      <c r="J4" s="31">
-        <f t="shared" ref="J4:J11" si="3">0.01*H4</f>
-        <v>0</v>
-      </c>
-      <c r="K4" s="31">
-        <f t="shared" ref="K4:K11" si="4">SUM(H4:J4)</f>
-        <v>0</v>
-      </c>
-      <c r="L4" s="30">
-        <f t="shared" ref="L4:L11" si="5">K4*60*24/10^6</f>
-        <v>0</v>
-      </c>
-      <c r="M4" s="31">
-        <f t="shared" ref="M4:M11" si="6">L4*365</f>
-        <v>0</v>
-      </c>
-      <c r="N4" s="31">
-        <f t="shared" ref="N4:N11" si="7">M4*D4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A5" s="26" t="s">
+      <c r="K4" s="59">
+        <f t="shared" ref="K4:K11" si="3">0.001*J4*H4</f>
+        <v>568.66647711117434</v>
+      </c>
+      <c r="L4" s="59">
+        <f t="shared" ref="L4:L11" si="4">K4/(I4-1)</f>
+        <v>284.33323855558717</v>
+      </c>
+      <c r="M4" s="59">
+        <f t="shared" ref="M4:M11" si="5">0.01*K4</f>
+        <v>5.6866647711117437</v>
+      </c>
+      <c r="N4" s="59">
+        <f t="shared" ref="N4:N11" si="6">SUM(K4:M4)</f>
+        <v>858.68638043787325</v>
+      </c>
+      <c r="O4" s="60">
+        <f t="shared" ref="O4:O11" si="7">N4*60*24/10^6</f>
+        <v>1.2365083878305374</v>
+      </c>
+      <c r="P4" s="59">
+        <f t="shared" ref="P4:P11" si="8">O4*365</f>
+        <v>451.32556155814615</v>
+      </c>
+      <c r="Q4" s="59">
+        <f t="shared" ref="Q4:Q11" si="9">P4*G4</f>
+        <v>361.06044924651695</v>
+      </c>
+      <c r="R4" s="67">
+        <v>5.5</v>
+      </c>
+      <c r="S4" s="79">
+        <f>(Q4*(10^3))*$R$4</f>
+        <v>1985832.4708558433</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" s="39"/>
+      <c r="B5" s="55"/>
+      <c r="C5" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" s="1">
+        <v>100</v>
+      </c>
+      <c r="E5" s="67"/>
+      <c r="F5" s="82"/>
+      <c r="G5" s="57">
+        <v>0.6</v>
+      </c>
+      <c r="H5" s="1">
+        <v>20</v>
+      </c>
+      <c r="I5" s="1">
+        <v>3</v>
+      </c>
+      <c r="J5" s="58">
+        <f t="shared" si="2"/>
+        <v>28433.323855558716</v>
+      </c>
+      <c r="K5" s="59">
+        <f t="shared" si="3"/>
+        <v>568.66647711117434</v>
+      </c>
+      <c r="L5" s="59">
+        <f t="shared" si="4"/>
+        <v>284.33323855558717</v>
+      </c>
+      <c r="M5" s="59">
+        <f t="shared" si="5"/>
+        <v>5.6866647711117437</v>
+      </c>
+      <c r="N5" s="59">
+        <f t="shared" si="6"/>
+        <v>858.68638043787325</v>
+      </c>
+      <c r="O5" s="60">
+        <f t="shared" si="7"/>
+        <v>1.2365083878305374</v>
+      </c>
+      <c r="P5" s="59">
+        <f t="shared" si="8"/>
+        <v>451.32556155814615</v>
+      </c>
+      <c r="Q5" s="59">
+        <f t="shared" si="9"/>
+        <v>270.7953369348877</v>
+      </c>
+      <c r="R5" s="67"/>
+      <c r="S5" s="79">
+        <f>(Q5*(10^3))*$R$4</f>
+        <v>1489374.3531418822</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" s="39" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="54" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B5" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="C5" s="26">
+      <c r="D6" s="2">
         <v>100</v>
       </c>
-      <c r="D5" s="29">
+      <c r="E6" s="65">
+        <v>0.13</v>
+      </c>
+      <c r="F6" s="81">
+        <f t="shared" ref="F6" si="10">D6*1000*365*E6</f>
+        <v>4745000</v>
+      </c>
+      <c r="G6" s="20">
+        <v>0.8</v>
+      </c>
+      <c r="H6" s="49">
+        <v>15</v>
+      </c>
+      <c r="I6" s="49">
+        <v>3</v>
+      </c>
+      <c r="J6" s="21">
+        <f t="shared" si="2"/>
+        <v>28433.323855558716</v>
+      </c>
+      <c r="K6" s="22">
+        <f t="shared" si="3"/>
+        <v>426.4998578333807</v>
+      </c>
+      <c r="L6" s="22">
+        <f t="shared" si="4"/>
+        <v>213.24992891669035</v>
+      </c>
+      <c r="M6" s="22">
+        <f t="shared" si="5"/>
+        <v>4.2649985783338069</v>
+      </c>
+      <c r="N6" s="22">
+        <f t="shared" si="6"/>
+        <v>644.01478532840486</v>
+      </c>
+      <c r="O6" s="23">
+        <f t="shared" si="7"/>
+        <v>0.927381290872903</v>
+      </c>
+      <c r="P6" s="22">
+        <f t="shared" si="8"/>
+        <v>338.49417116860957</v>
+      </c>
+      <c r="Q6" s="66">
+        <f t="shared" si="9"/>
+        <v>270.79533693488764</v>
+      </c>
+      <c r="R6" s="65">
+        <v>3.5</v>
+      </c>
+      <c r="S6" s="78">
+        <f>(Q6*(10^3))*$R$6</f>
+        <v>947783.67927210673</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" s="39"/>
+      <c r="B7" s="54"/>
+      <c r="C7" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D7" s="2">
+        <v>100</v>
+      </c>
+      <c r="E7" s="65"/>
+      <c r="F7" s="81"/>
+      <c r="G7" s="20">
         <v>0.6</v>
       </c>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="33">
-        <f t="shared" si="0"/>
+      <c r="H7" s="49">
+        <v>15</v>
+      </c>
+      <c r="I7" s="49">
+        <v>3</v>
+      </c>
+      <c r="J7" s="21">
+        <f t="shared" si="2"/>
         <v>28433.323855558716</v>
       </c>
-      <c r="H5" s="31">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I5" s="31">
+      <c r="K7" s="22">
+        <f t="shared" si="3"/>
+        <v>426.4998578333807</v>
+      </c>
+      <c r="L7" s="22">
+        <f t="shared" si="4"/>
+        <v>213.24992891669035</v>
+      </c>
+      <c r="M7" s="22">
+        <f t="shared" si="5"/>
+        <v>4.2649985783338069</v>
+      </c>
+      <c r="N7" s="22">
+        <f t="shared" si="6"/>
+        <v>644.01478532840486</v>
+      </c>
+      <c r="O7" s="23">
+        <f t="shared" si="7"/>
+        <v>0.927381290872903</v>
+      </c>
+      <c r="P7" s="22">
+        <f t="shared" si="8"/>
+        <v>338.49417116860957</v>
+      </c>
+      <c r="Q7" s="66">
+        <f t="shared" si="9"/>
+        <v>203.09650270116575</v>
+      </c>
+      <c r="R7" s="65"/>
+      <c r="S7" s="78">
+        <f>(Q7*(10^3))*$R$6</f>
+        <v>710837.75945408014</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A8" s="39" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="55" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" s="1">
+        <v>100</v>
+      </c>
+      <c r="E8" s="67">
+        <v>0.3</v>
+      </c>
+      <c r="F8" s="82">
+        <f t="shared" ref="F8" si="11">D8*1000*365*E8</f>
+        <v>10950000</v>
+      </c>
+      <c r="G8" s="57">
+        <v>0.8</v>
+      </c>
+      <c r="H8" s="1">
+        <v>20</v>
+      </c>
+      <c r="I8" s="1">
+        <v>3</v>
+      </c>
+      <c r="J8" s="58">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J5" s="31">
+        <v>28433.323855558716</v>
+      </c>
+      <c r="K8" s="59">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="K5" s="31">
+        <v>568.66647711117434</v>
+      </c>
+      <c r="L8" s="59">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="L5" s="30">
+        <v>284.33323855558717</v>
+      </c>
+      <c r="M8" s="59">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="M5" s="31">
+        <v>5.6866647711117437</v>
+      </c>
+      <c r="N8" s="59">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N5" s="31">
+        <v>858.68638043787325</v>
+      </c>
+      <c r="O8" s="60">
         <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A6" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="B6" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="C6" s="26">
+        <v>1.2365083878305374</v>
+      </c>
+      <c r="P8" s="59">
+        <f t="shared" si="8"/>
+        <v>451.32556155814615</v>
+      </c>
+      <c r="Q8" s="59">
+        <f t="shared" si="9"/>
+        <v>361.06044924651695</v>
+      </c>
+      <c r="R8" s="67">
+        <v>11.5</v>
+      </c>
+      <c r="S8" s="79">
+        <f>(Q8*(10^3))*$R$8</f>
+        <v>4152195.1663349452</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A9" s="39"/>
+      <c r="B9" s="55"/>
+      <c r="C9" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D9" s="1">
         <v>100</v>
       </c>
-      <c r="D6" s="29">
+      <c r="E9" s="67"/>
+      <c r="F9" s="82"/>
+      <c r="G9" s="57">
+        <v>0.6</v>
+      </c>
+      <c r="H9" s="1">
+        <v>20</v>
+      </c>
+      <c r="I9" s="1">
+        <v>3</v>
+      </c>
+      <c r="J9" s="58">
+        <f t="shared" si="2"/>
+        <v>28433.323855558716</v>
+      </c>
+      <c r="K9" s="59">
+        <f t="shared" si="3"/>
+        <v>568.66647711117434</v>
+      </c>
+      <c r="L9" s="59">
+        <f t="shared" si="4"/>
+        <v>284.33323855558717</v>
+      </c>
+      <c r="M9" s="59">
+        <f t="shared" si="5"/>
+        <v>5.6866647711117437</v>
+      </c>
+      <c r="N9" s="59">
+        <f t="shared" si="6"/>
+        <v>858.68638043787325</v>
+      </c>
+      <c r="O9" s="60">
+        <f t="shared" si="7"/>
+        <v>1.2365083878305374</v>
+      </c>
+      <c r="P9" s="59">
+        <f t="shared" si="8"/>
+        <v>451.32556155814615</v>
+      </c>
+      <c r="Q9" s="59">
+        <f t="shared" si="9"/>
+        <v>270.7953369348877</v>
+      </c>
+      <c r="R9" s="67"/>
+      <c r="S9" s="79">
+        <f>(Q9*(10^3))*$R$8</f>
+        <v>3114146.3747512084</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A10" s="39" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="54" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" s="2">
+        <v>100</v>
+      </c>
+      <c r="E10" s="65">
+        <v>0.12</v>
+      </c>
+      <c r="F10" s="81">
+        <f t="shared" ref="F10" si="12">D10*1000*365*E10</f>
+        <v>4380000</v>
+      </c>
+      <c r="G10" s="20">
         <v>0.8</v>
       </c>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="33">
-        <f t="shared" si="0"/>
+      <c r="H10" s="49">
+        <v>10</v>
+      </c>
+      <c r="I10" s="49">
+        <v>4</v>
+      </c>
+      <c r="J10" s="21">
+        <f t="shared" si="2"/>
         <v>28433.323855558716</v>
       </c>
-      <c r="H6" s="31">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I6" s="31">
+      <c r="K10" s="22">
+        <f t="shared" si="3"/>
+        <v>284.33323855558717</v>
+      </c>
+      <c r="L10" s="22">
+        <f t="shared" si="4"/>
+        <v>94.777746185195724</v>
+      </c>
+      <c r="M10" s="22">
+        <f t="shared" si="5"/>
+        <v>2.8433323855558719</v>
+      </c>
+      <c r="N10" s="22">
+        <f t="shared" si="6"/>
+        <v>381.95431712633876</v>
+      </c>
+      <c r="O10" s="23">
+        <f t="shared" si="7"/>
+        <v>0.55001421666192785</v>
+      </c>
+      <c r="P10" s="22">
+        <f t="shared" si="8"/>
+        <v>200.75518908160367</v>
+      </c>
+      <c r="Q10" s="66">
+        <f t="shared" si="9"/>
+        <v>160.60415126528295</v>
+      </c>
+      <c r="R10" s="65">
+        <v>5.5</v>
+      </c>
+      <c r="S10" s="78">
+        <f>(Q10*(10^3))*$R$10</f>
+        <v>883322.8319590562</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="39"/>
+      <c r="B11" s="73"/>
+      <c r="C11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="D11" s="11">
+        <v>100</v>
+      </c>
+      <c r="E11" s="74"/>
+      <c r="F11" s="83"/>
+      <c r="G11" s="24">
+        <v>0.6</v>
+      </c>
+      <c r="H11" s="50">
+        <v>10</v>
+      </c>
+      <c r="I11" s="50">
+        <v>4</v>
+      </c>
+      <c r="J11" s="25">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J6" s="31">
+        <v>28433.323855558716</v>
+      </c>
+      <c r="K11" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="K6" s="31">
+        <v>284.33323855558717</v>
+      </c>
+      <c r="L11" s="26">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="L6" s="30">
+        <v>94.777746185195724</v>
+      </c>
+      <c r="M11" s="26">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="M6" s="31">
+        <v>2.8433323855558719</v>
+      </c>
+      <c r="N11" s="26">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N6" s="31">
+        <v>381.95431712633876</v>
+      </c>
+      <c r="O11" s="27">
         <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A7" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="B7" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="C7" s="26">
-        <v>100</v>
-      </c>
-      <c r="D7" s="29">
-        <v>0.6</v>
-      </c>
-      <c r="E7" s="34"/>
-      <c r="F7" s="34"/>
-      <c r="G7" s="33">
-        <f t="shared" si="0"/>
-        <v>28433.323855558716</v>
-      </c>
-      <c r="H7" s="31">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I7" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J7" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="K7" s="31">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="L7" s="30">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="M7" s="31">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N7" s="31">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A8" s="26" t="s">
-        <v>69</v>
-      </c>
-      <c r="B8" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="C8" s="26">
-        <v>100</v>
-      </c>
-      <c r="D8" s="29">
-        <v>0.8</v>
-      </c>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="33">
-        <f t="shared" si="0"/>
-        <v>28433.323855558716</v>
-      </c>
-      <c r="H8" s="31">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I8" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J8" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="K8" s="31">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="L8" s="30">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="M8" s="31">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N8" s="31">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A9" s="26" t="s">
-        <v>69</v>
-      </c>
-      <c r="B9" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="C9" s="26">
-        <v>100</v>
-      </c>
-      <c r="D9" s="29">
-        <v>0.6</v>
-      </c>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34"/>
-      <c r="G9" s="33">
-        <f t="shared" si="0"/>
-        <v>28433.323855558716</v>
-      </c>
-      <c r="H9" s="31">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I9" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J9" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="K9" s="31">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="L9" s="30">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="M9" s="31">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N9" s="31">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A10" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="B10" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="C10" s="26">
-        <v>100</v>
-      </c>
-      <c r="D10" s="29">
-        <v>0.8</v>
-      </c>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="33">
-        <f t="shared" si="0"/>
-        <v>28433.323855558716</v>
-      </c>
-      <c r="H10" s="31">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I10" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J10" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="K10" s="31">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="L10" s="30">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="M10" s="31">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N10" s="31">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A11" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="B11" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="C11" s="26">
-        <v>100</v>
-      </c>
-      <c r="D11" s="29">
-        <v>0.6</v>
-      </c>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="33">
-        <f t="shared" si="0"/>
-        <v>28433.323855558716</v>
-      </c>
-      <c r="H11" s="31">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I11" s="31">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J11" s="31">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="K11" s="31">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="L11" s="30">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="M11" s="31">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N11" s="31">
-        <f t="shared" si="7"/>
-        <v>0</v>
+        <v>0.55001421666192785</v>
+      </c>
+      <c r="P11" s="26">
+        <f t="shared" si="8"/>
+        <v>200.75518908160367</v>
+      </c>
+      <c r="Q11" s="75">
+        <f t="shared" si="9"/>
+        <v>120.4531134489622</v>
+      </c>
+      <c r="R11" s="74"/>
+      <c r="S11" s="78">
+        <f>(Q11*(10^3))*$R$10</f>
+        <v>662492.12396929215</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="25">
+    <mergeCell ref="R10:R11"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="R2:R3"/>
+    <mergeCell ref="R4:R5"/>
+    <mergeCell ref="R6:R7"/>
+    <mergeCell ref="R8:R9"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A11"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>

</xml_diff>

<commit_message>
Update Excel data file with new Total Impact score
</commit_message>
<xml_diff>
--- a/Final.Project.Data.xlsx
+++ b/Final.Project.Data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gmste\CES Dropbox\Thomas Sowden\PC (2)\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://colostate-my.sharepoint.com/personal/c829804536_colostate_edu/Documents/Microsoft Teams Chat Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DFB53C7-84D2-4D09-BFED-E70142B3A2AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="728" documentId="13_ncr:1_{143D07AB-F20C-4929-836A-E19FFE3DAE4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB9A80D9-FA40-4C6B-A44A-393028FD13A9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{83A2F5A8-6268-4F4A-A0FD-FC6B17854872}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="50">
   <si>
     <t>Climate Type</t>
   </si>
@@ -187,6 +187,15 @@
     <t>Annual CO2 (metric tons)</t>
   </si>
   <si>
+    <t>Carbon Price ($/ metric ton)</t>
+  </si>
+  <si>
+    <t>Annual Carbon Cost ($)</t>
+  </si>
+  <si>
+    <t>Normalized Carbon Cost (Scale: 0-1)</t>
+  </si>
+  <si>
     <t>Climate Adjusted Water Use (gallons/year)</t>
   </si>
   <si>
@@ -202,6 +211,9 @@
     <t>Monthly Precip</t>
   </si>
   <si>
+    <t>Total Impact</t>
+  </si>
+  <si>
     <t>Stress</t>
   </si>
   <si>
@@ -209,9 +221,6 @@
   </si>
   <si>
     <t>Note - The Avg Annual Precip values were taken from the official 1991–2020 U.S. Climate Normals (NOAA), which are 30-year averages calculated from thousands of weather stations.</t>
-  </si>
-  <si>
-    <t>Site Selection</t>
   </si>
 </sst>
 </file>
@@ -223,7 +232,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -258,8 +267,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -308,14 +324,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.749992370372631"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="25">
+  <borders count="48">
     <border>
       <left/>
       <right/>
@@ -606,15 +616,28 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </left>
       <right/>
       <top style="medium">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="medium">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -622,35 +645,305 @@
       <left/>
       <right/>
       <top style="medium">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="medium">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="medium">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="medium">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
       <top/>
       <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -659,7 +952,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -700,9 +993,6 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -739,16 +1029,100 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -763,6 +1137,18 @@
     <xf numFmtId="1" fontId="0" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -781,6 +1167,12 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -799,18 +1191,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -834,30 +1214,6 @@
     </xf>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -865,16 +1221,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -889,6 +1242,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -901,23 +1275,23 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="47" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1208,6 +1582,53 @@
         </a:p>
       </xdr:txBody>
     </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>85725</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>314325</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5BA5C43C-AF5E-C948-7DE6-23D169CA0D29}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{6211333C-F9B8-9317-E79F-DCBF79044BD3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="800100" y="10153650"/>
+          <a:ext cx="10344150" cy="2714625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -1533,9 +1954,9 @@
   <dimension ref="B1:W22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="8.7109375" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" customWidth="1"/>
-    <col min="4" max="4" width="8.85546875" customWidth="1"/>
+    <col min="2" max="2" width="0.42578125" customWidth="1"/>
+    <col min="3" max="3" width="1.140625" customWidth="1"/>
+    <col min="4" max="4" width="3.42578125" customWidth="1"/>
     <col min="5" max="5" width="18.42578125" customWidth="1"/>
     <col min="6" max="6" width="13.85546875" style="3" customWidth="1"/>
     <col min="7" max="7" width="16.5703125" style="3" customWidth="1"/>
@@ -1545,7 +1966,8 @@
     <col min="11" max="11" width="10.5703125" style="4" customWidth="1"/>
     <col min="12" max="13" width="10.5703125" style="3" customWidth="1"/>
     <col min="14" max="14" width="14.28515625" style="5" customWidth="1"/>
-    <col min="15" max="17" width="10.5703125" style="3" customWidth="1"/>
+    <col min="15" max="16" width="10.5703125" style="3" customWidth="1"/>
+    <col min="17" max="17" width="13.28515625" style="3" customWidth="1"/>
     <col min="18" max="18" width="14.28515625" style="3" customWidth="1"/>
     <col min="19" max="19" width="10.5703125" style="3" customWidth="1"/>
     <col min="20" max="20" width="13.42578125" style="3" customWidth="1"/>
@@ -1554,40 +1976,18 @@
     <col min="23" max="23" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E1" s="84" t="s">
-        <v>46</v>
-      </c>
-      <c r="F1" s="85"/>
-      <c r="G1" s="85"/>
-      <c r="H1" s="85"/>
-      <c r="I1" s="85"/>
-      <c r="J1" s="85"/>
-      <c r="K1" s="85"/>
-      <c r="L1" s="85"/>
-      <c r="M1" s="85"/>
-      <c r="N1" s="85"/>
-      <c r="O1" s="85"/>
-      <c r="P1" s="85"/>
-      <c r="Q1" s="85"/>
-      <c r="R1" s="85"/>
-      <c r="S1" s="85"/>
-      <c r="T1" s="85"/>
-      <c r="U1" s="85"/>
-      <c r="V1" s="85"/>
-      <c r="W1" s="86"/>
-    </row>
+    <row r="1" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:23" s="2" customFormat="1" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="26" t="s">
+      <c r="F2" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="25" t="s">
+      <c r="G2" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="25" t="s">
+      <c r="H2" s="24" t="s">
         <v>3</v>
       </c>
       <c r="I2" s="10" t="s">
@@ -1637,96 +2037,96 @@
       </c>
     </row>
     <row r="3" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="E3" s="64" t="s">
+      <c r="E3" s="109" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="75" t="s">
+      <c r="F3" s="95" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="47" t="s">
+      <c r="G3" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="47">
+      <c r="H3" s="72">
         <v>100</v>
       </c>
-      <c r="I3" s="61">
+      <c r="I3" s="62">
         <v>0.13</v>
       </c>
-      <c r="J3" s="51">
+      <c r="J3" s="80">
         <f>H3*1000*365*I3</f>
         <v>4745000</v>
       </c>
-      <c r="K3" s="41">
+      <c r="K3" s="74">
         <f>IF(G3=B5,0.8,0.6)</f>
         <v>0.8</v>
       </c>
-      <c r="L3" s="43">
+      <c r="L3" s="76">
         <f>70-55</f>
         <v>15</v>
       </c>
-      <c r="M3" s="43">
+      <c r="M3" s="76">
         <v>4</v>
       </c>
-      <c r="N3" s="55">
+      <c r="N3" s="84">
         <f>H3*1000/3.517</f>
         <v>28433.323855558716</v>
       </c>
-      <c r="O3" s="35">
+      <c r="O3" s="66">
         <f>0.001*N3*L3</f>
         <v>426.4998578333807</v>
       </c>
-      <c r="P3" s="35">
+      <c r="P3" s="66">
         <f>O3/(M3-1)</f>
         <v>142.16661927779356</v>
       </c>
-      <c r="Q3" s="35">
+      <c r="Q3" s="66">
         <f>0.01*O3</f>
         <v>4.2649985783338069</v>
       </c>
-      <c r="R3" s="35">
+      <c r="R3" s="66">
         <f>SUM(O3:Q3)</f>
         <v>572.93147568950803</v>
       </c>
-      <c r="S3" s="37">
+      <c r="S3" s="68">
         <f>R3*60*24/10^6</f>
         <v>0.8250213249928916</v>
       </c>
-      <c r="T3" s="35">
+      <c r="T3" s="66">
         <f>S3*365</f>
         <v>301.13278362240544</v>
       </c>
-      <c r="U3" s="31">
+      <c r="U3" s="58">
         <f>T3*K3</f>
         <v>240.90622689792437</v>
       </c>
-      <c r="V3" s="61">
+      <c r="V3" s="62">
         <v>4.9000000000000004</v>
       </c>
-      <c r="W3" s="27">
+      <c r="W3" s="54">
         <f>(U3*(10^3))*$V$3</f>
         <v>1180440.5117998295</v>
       </c>
     </row>
     <row r="4" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E4" s="63"/>
-      <c r="F4" s="76"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="48"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="52"/>
-      <c r="K4" s="42"/>
-      <c r="L4" s="44"/>
-      <c r="M4" s="44"/>
-      <c r="N4" s="56"/>
-      <c r="O4" s="36"/>
-      <c r="P4" s="36"/>
-      <c r="Q4" s="36"/>
-      <c r="R4" s="36"/>
-      <c r="S4" s="38"/>
-      <c r="T4" s="36"/>
-      <c r="U4" s="32"/>
-      <c r="V4" s="62"/>
-      <c r="W4" s="28"/>
+      <c r="E4" s="108"/>
+      <c r="F4" s="96"/>
+      <c r="G4" s="73"/>
+      <c r="H4" s="73"/>
+      <c r="I4" s="63"/>
+      <c r="J4" s="81"/>
+      <c r="K4" s="75"/>
+      <c r="L4" s="77"/>
+      <c r="M4" s="77"/>
+      <c r="N4" s="85"/>
+      <c r="O4" s="67"/>
+      <c r="P4" s="67"/>
+      <c r="Q4" s="67"/>
+      <c r="R4" s="67"/>
+      <c r="S4" s="69"/>
+      <c r="T4" s="67"/>
+      <c r="U4" s="59"/>
+      <c r="V4" s="63"/>
+      <c r="W4" s="55"/>
     </row>
     <row r="5" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
@@ -1735,71 +2135,71 @@
       <c r="C5">
         <v>50</v>
       </c>
-      <c r="E5" s="63" t="s">
+      <c r="E5" s="108" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="79" t="s">
+      <c r="F5" s="106" t="s">
         <v>23</v>
       </c>
-      <c r="G5" s="49" t="s">
+      <c r="G5" s="97" t="s">
         <v>21</v>
       </c>
-      <c r="H5" s="49">
+      <c r="H5" s="97">
         <v>100</v>
       </c>
-      <c r="I5" s="59">
+      <c r="I5" s="64">
         <v>0.12</v>
       </c>
-      <c r="J5" s="53">
+      <c r="J5" s="82">
         <f>H5*1000*365*I5</f>
         <v>4380000</v>
       </c>
-      <c r="K5" s="77">
+      <c r="K5" s="104">
         <f t="shared" ref="K5" si="0">IF(G5=B7,0.8,0.6)</f>
         <v>0.6</v>
       </c>
-      <c r="L5" s="45">
+      <c r="L5" s="78">
         <v>20</v>
       </c>
-      <c r="M5" s="45">
+      <c r="M5" s="78">
         <v>3</v>
       </c>
-      <c r="N5" s="57">
+      <c r="N5" s="86">
         <f t="shared" ref="N5:N11" si="1">H5*1000/3.517</f>
         <v>28433.323855558716</v>
       </c>
-      <c r="O5" s="33">
+      <c r="O5" s="60">
         <f t="shared" ref="O5:O11" si="2">0.001*N5*L5</f>
         <v>568.66647711117434</v>
       </c>
-      <c r="P5" s="33">
+      <c r="P5" s="60">
         <f t="shared" ref="P5:P11" si="3">O5/(M5-1)</f>
         <v>284.33323855558717</v>
       </c>
-      <c r="Q5" s="33">
+      <c r="Q5" s="60">
         <f t="shared" ref="Q5:Q11" si="4">0.01*O5</f>
         <v>5.6866647711117437</v>
       </c>
-      <c r="R5" s="33">
+      <c r="R5" s="60">
         <f t="shared" ref="R5:R11" si="5">SUM(O5:Q5)</f>
         <v>858.68638043787325</v>
       </c>
-      <c r="S5" s="39">
+      <c r="S5" s="70">
         <f t="shared" ref="S5:S11" si="6">R5*60*24/10^6</f>
         <v>1.2365083878305374</v>
       </c>
-      <c r="T5" s="33">
+      <c r="T5" s="60">
         <f t="shared" ref="T5:T11" si="7">S5*365</f>
         <v>451.32556155814615</v>
       </c>
-      <c r="U5" s="33">
+      <c r="U5" s="60">
         <f t="shared" ref="U5:U11" si="8">T5*K5</f>
         <v>270.7953369348877</v>
       </c>
-      <c r="V5" s="59">
+      <c r="V5" s="64">
         <v>5.5</v>
       </c>
-      <c r="W5" s="29">
+      <c r="W5" s="56">
         <f>(U5*(10^3))*$V$5</f>
         <v>1489374.3531418822</v>
       </c>
@@ -1811,95 +2211,95 @@
       <c r="C6">
         <v>100</v>
       </c>
-      <c r="E6" s="63"/>
-      <c r="F6" s="80"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="50"/>
-      <c r="I6" s="60"/>
-      <c r="J6" s="54"/>
-      <c r="K6" s="78"/>
-      <c r="L6" s="46"/>
-      <c r="M6" s="46"/>
-      <c r="N6" s="58"/>
-      <c r="O6" s="34"/>
-      <c r="P6" s="34"/>
-      <c r="Q6" s="34"/>
-      <c r="R6" s="34"/>
-      <c r="S6" s="40"/>
-      <c r="T6" s="34"/>
-      <c r="U6" s="34"/>
-      <c r="V6" s="60"/>
-      <c r="W6" s="30"/>
+      <c r="E6" s="108"/>
+      <c r="F6" s="107"/>
+      <c r="G6" s="98"/>
+      <c r="H6" s="98"/>
+      <c r="I6" s="65"/>
+      <c r="J6" s="83"/>
+      <c r="K6" s="105"/>
+      <c r="L6" s="79"/>
+      <c r="M6" s="79"/>
+      <c r="N6" s="87"/>
+      <c r="O6" s="61"/>
+      <c r="P6" s="61"/>
+      <c r="Q6" s="61"/>
+      <c r="R6" s="61"/>
+      <c r="S6" s="71"/>
+      <c r="T6" s="61"/>
+      <c r="U6" s="61"/>
+      <c r="V6" s="65"/>
+      <c r="W6" s="57"/>
     </row>
     <row r="7" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C7">
         <v>150</v>
       </c>
-      <c r="E7" s="63" t="s">
+      <c r="E7" s="108" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="75" t="s">
+      <c r="F7" s="95" t="s">
         <v>26</v>
       </c>
-      <c r="G7" s="47" t="s">
+      <c r="G7" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="H7" s="47">
+      <c r="H7" s="72">
         <v>100</v>
       </c>
-      <c r="I7" s="61">
+      <c r="I7" s="62">
         <v>0.13</v>
       </c>
-      <c r="J7" s="51">
+      <c r="J7" s="80">
         <f>H7*1000*365*I7</f>
         <v>4745000</v>
       </c>
-      <c r="K7" s="41">
+      <c r="K7" s="74">
         <f t="shared" ref="K7" si="9">IF(G7=B9,0.8,0.6)</f>
         <v>0.6</v>
       </c>
-      <c r="L7" s="43">
+      <c r="L7" s="76">
         <v>15</v>
       </c>
-      <c r="M7" s="43">
+      <c r="M7" s="76">
         <v>3</v>
       </c>
-      <c r="N7" s="55">
+      <c r="N7" s="84">
         <f t="shared" si="1"/>
         <v>28433.323855558716</v>
       </c>
-      <c r="O7" s="35">
+      <c r="O7" s="66">
         <f t="shared" si="2"/>
         <v>426.4998578333807</v>
       </c>
-      <c r="P7" s="35">
+      <c r="P7" s="66">
         <f t="shared" si="3"/>
         <v>213.24992891669035</v>
       </c>
-      <c r="Q7" s="35">
+      <c r="Q7" s="66">
         <f t="shared" si="4"/>
         <v>4.2649985783338069</v>
       </c>
-      <c r="R7" s="35">
+      <c r="R7" s="66">
         <f t="shared" si="5"/>
         <v>644.01478532840486</v>
       </c>
-      <c r="S7" s="37">
+      <c r="S7" s="68">
         <f t="shared" si="6"/>
         <v>0.927381290872903</v>
       </c>
-      <c r="T7" s="35">
+      <c r="T7" s="66">
         <f t="shared" si="7"/>
         <v>338.49417116860957</v>
       </c>
-      <c r="U7" s="31">
+      <c r="U7" s="58">
         <f t="shared" si="8"/>
         <v>203.09650270116575</v>
       </c>
-      <c r="V7" s="61">
+      <c r="V7" s="62">
         <v>3.5</v>
       </c>
-      <c r="W7" s="27">
+      <c r="W7" s="54">
         <f>(U7*(10^3))*$V$7</f>
         <v>710837.75945408014</v>
       </c>
@@ -1911,25 +2311,25 @@
       <c r="C8">
         <v>200</v>
       </c>
-      <c r="E8" s="63"/>
-      <c r="F8" s="76"/>
-      <c r="G8" s="48"/>
-      <c r="H8" s="48"/>
-      <c r="I8" s="62"/>
-      <c r="J8" s="52"/>
-      <c r="K8" s="42"/>
-      <c r="L8" s="44"/>
-      <c r="M8" s="44"/>
-      <c r="N8" s="56"/>
-      <c r="O8" s="36"/>
-      <c r="P8" s="36"/>
-      <c r="Q8" s="36"/>
-      <c r="R8" s="36"/>
-      <c r="S8" s="38"/>
-      <c r="T8" s="36"/>
-      <c r="U8" s="32"/>
-      <c r="V8" s="62"/>
-      <c r="W8" s="28"/>
+      <c r="E8" s="108"/>
+      <c r="F8" s="96"/>
+      <c r="G8" s="73"/>
+      <c r="H8" s="73"/>
+      <c r="I8" s="63"/>
+      <c r="J8" s="81"/>
+      <c r="K8" s="75"/>
+      <c r="L8" s="77"/>
+      <c r="M8" s="77"/>
+      <c r="N8" s="85"/>
+      <c r="O8" s="67"/>
+      <c r="P8" s="67"/>
+      <c r="Q8" s="67"/>
+      <c r="R8" s="67"/>
+      <c r="S8" s="69"/>
+      <c r="T8" s="67"/>
+      <c r="U8" s="59"/>
+      <c r="V8" s="63"/>
+      <c r="W8" s="55"/>
     </row>
     <row r="9" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="8">
@@ -1938,71 +2338,71 @@
       <c r="C9">
         <v>250</v>
       </c>
-      <c r="E9" s="63" t="s">
+      <c r="E9" s="108" t="s">
         <v>27</v>
       </c>
-      <c r="F9" s="79" t="s">
+      <c r="F9" s="106" t="s">
         <v>28</v>
       </c>
-      <c r="G9" s="49" t="s">
+      <c r="G9" s="97" t="s">
         <v>21</v>
       </c>
-      <c r="H9" s="49">
+      <c r="H9" s="97">
         <v>100</v>
       </c>
-      <c r="I9" s="59">
+      <c r="I9" s="64">
         <v>0.3</v>
       </c>
-      <c r="J9" s="53">
+      <c r="J9" s="82">
         <f>H9*1000*365*I9</f>
         <v>10950000</v>
       </c>
-      <c r="K9" s="77">
+      <c r="K9" s="104">
         <f t="shared" ref="K9" si="10">IF(G9=B11,0.8,0.6)</f>
         <v>0.6</v>
       </c>
-      <c r="L9" s="45">
+      <c r="L9" s="78">
         <v>20</v>
       </c>
-      <c r="M9" s="45">
+      <c r="M9" s="78">
         <v>3</v>
       </c>
-      <c r="N9" s="57">
+      <c r="N9" s="86">
         <f t="shared" si="1"/>
         <v>28433.323855558716</v>
       </c>
-      <c r="O9" s="33">
+      <c r="O9" s="60">
         <f t="shared" si="2"/>
         <v>568.66647711117434</v>
       </c>
-      <c r="P9" s="33">
+      <c r="P9" s="60">
         <f t="shared" si="3"/>
         <v>284.33323855558717</v>
       </c>
-      <c r="Q9" s="33">
+      <c r="Q9" s="60">
         <f t="shared" si="4"/>
         <v>5.6866647711117437</v>
       </c>
-      <c r="R9" s="33">
+      <c r="R9" s="60">
         <f t="shared" si="5"/>
         <v>858.68638043787325</v>
       </c>
-      <c r="S9" s="39">
+      <c r="S9" s="70">
         <f t="shared" si="6"/>
         <v>1.2365083878305374</v>
       </c>
-      <c r="T9" s="33">
+      <c r="T9" s="60">
         <f t="shared" si="7"/>
         <v>451.32556155814615</v>
       </c>
-      <c r="U9" s="33">
+      <c r="U9" s="60">
         <f t="shared" si="8"/>
         <v>270.7953369348877</v>
       </c>
-      <c r="V9" s="59">
+      <c r="V9" s="64">
         <v>11.5</v>
       </c>
-      <c r="W9" s="29">
+      <c r="W9" s="56">
         <f>(U9*(10^3))*$V$9</f>
         <v>3114146.3747512084</v>
       </c>
@@ -2011,95 +2411,95 @@
       <c r="C10">
         <v>300</v>
       </c>
-      <c r="E10" s="63"/>
-      <c r="F10" s="80"/>
-      <c r="G10" s="50"/>
-      <c r="H10" s="50"/>
-      <c r="I10" s="60"/>
-      <c r="J10" s="54"/>
-      <c r="K10" s="78"/>
-      <c r="L10" s="46"/>
-      <c r="M10" s="46"/>
-      <c r="N10" s="58"/>
-      <c r="O10" s="34"/>
-      <c r="P10" s="34"/>
-      <c r="Q10" s="34"/>
-      <c r="R10" s="34"/>
-      <c r="S10" s="40"/>
-      <c r="T10" s="34"/>
-      <c r="U10" s="34"/>
-      <c r="V10" s="60"/>
-      <c r="W10" s="30"/>
+      <c r="E10" s="108"/>
+      <c r="F10" s="107"/>
+      <c r="G10" s="98"/>
+      <c r="H10" s="98"/>
+      <c r="I10" s="65"/>
+      <c r="J10" s="83"/>
+      <c r="K10" s="105"/>
+      <c r="L10" s="79"/>
+      <c r="M10" s="79"/>
+      <c r="N10" s="87"/>
+      <c r="O10" s="61"/>
+      <c r="P10" s="61"/>
+      <c r="Q10" s="61"/>
+      <c r="R10" s="61"/>
+      <c r="S10" s="71"/>
+      <c r="T10" s="61"/>
+      <c r="U10" s="61"/>
+      <c r="V10" s="65"/>
+      <c r="W10" s="57"/>
     </row>
     <row r="11" spans="2:23" x14ac:dyDescent="0.25">
       <c r="C11">
         <v>350</v>
       </c>
-      <c r="E11" s="63" t="s">
+      <c r="E11" s="108" t="s">
         <v>29</v>
       </c>
-      <c r="F11" s="75" t="s">
+      <c r="F11" s="95" t="s">
         <v>30</v>
       </c>
-      <c r="G11" s="47" t="s">
+      <c r="G11" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="47">
+      <c r="H11" s="72">
         <v>100</v>
       </c>
-      <c r="I11" s="61">
+      <c r="I11" s="62">
         <v>0.12</v>
       </c>
-      <c r="J11" s="51">
+      <c r="J11" s="80">
         <f t="shared" ref="J11" si="11">H11*1000*365*I11</f>
         <v>4380000</v>
       </c>
-      <c r="K11" s="41">
+      <c r="K11" s="74">
         <f t="shared" ref="K11" si="12">IF(G11=B13,0.8,0.6)</f>
         <v>0.6</v>
       </c>
-      <c r="L11" s="43">
+      <c r="L11" s="76">
         <v>10</v>
       </c>
-      <c r="M11" s="43">
+      <c r="M11" s="76">
         <v>4</v>
       </c>
-      <c r="N11" s="55">
+      <c r="N11" s="84">
         <f t="shared" si="1"/>
         <v>28433.323855558716</v>
       </c>
-      <c r="O11" s="35">
+      <c r="O11" s="66">
         <f t="shared" si="2"/>
         <v>284.33323855558717</v>
       </c>
-      <c r="P11" s="35">
+      <c r="P11" s="66">
         <f t="shared" si="3"/>
         <v>94.777746185195724</v>
       </c>
-      <c r="Q11" s="35">
+      <c r="Q11" s="66">
         <f t="shared" si="4"/>
         <v>2.8433323855558719</v>
       </c>
-      <c r="R11" s="35">
+      <c r="R11" s="66">
         <f t="shared" si="5"/>
         <v>381.95431712633876</v>
       </c>
-      <c r="S11" s="37">
+      <c r="S11" s="68">
         <f t="shared" si="6"/>
         <v>0.55001421666192785</v>
       </c>
-      <c r="T11" s="35">
+      <c r="T11" s="66">
         <f t="shared" si="7"/>
         <v>200.75518908160367</v>
       </c>
-      <c r="U11" s="31">
+      <c r="U11" s="58">
         <f t="shared" si="8"/>
         <v>120.4531134489622</v>
       </c>
-      <c r="V11" s="61">
+      <c r="V11" s="62">
         <v>5.5</v>
       </c>
-      <c r="W11" s="27">
+      <c r="W11" s="54">
         <f>(U11*(10^3))*$V$11</f>
         <v>662492.12396929215</v>
       </c>
@@ -2108,129 +2508,158 @@
       <c r="C12">
         <v>400</v>
       </c>
-      <c r="E12" s="65"/>
-      <c r="F12" s="76"/>
-      <c r="G12" s="48"/>
-      <c r="H12" s="48"/>
-      <c r="I12" s="62"/>
-      <c r="J12" s="52"/>
-      <c r="K12" s="42"/>
-      <c r="L12" s="44"/>
-      <c r="M12" s="44"/>
-      <c r="N12" s="56"/>
-      <c r="O12" s="36"/>
-      <c r="P12" s="36"/>
-      <c r="Q12" s="36"/>
-      <c r="R12" s="36"/>
-      <c r="S12" s="38"/>
-      <c r="T12" s="36"/>
-      <c r="U12" s="32"/>
-      <c r="V12" s="62"/>
-      <c r="W12" s="28"/>
+      <c r="E12" s="110"/>
+      <c r="F12" s="96"/>
+      <c r="G12" s="73"/>
+      <c r="H12" s="73"/>
+      <c r="I12" s="63"/>
+      <c r="J12" s="81"/>
+      <c r="K12" s="75"/>
+      <c r="L12" s="77"/>
+      <c r="M12" s="77"/>
+      <c r="N12" s="85"/>
+      <c r="O12" s="67"/>
+      <c r="P12" s="67"/>
+      <c r="Q12" s="67"/>
+      <c r="R12" s="67"/>
+      <c r="S12" s="69"/>
+      <c r="T12" s="67"/>
+      <c r="U12" s="59"/>
+      <c r="V12" s="63"/>
+      <c r="W12" s="55"/>
     </row>
-    <row r="13" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:23" x14ac:dyDescent="0.25">
       <c r="C13">
         <v>450</v>
       </c>
     </row>
-    <row r="14" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:23" x14ac:dyDescent="0.25">
       <c r="C14">
         <v>550</v>
       </c>
-      <c r="E14" s="81" t="s">
+      <c r="E14" s="51" t="s">
         <v>31</v>
       </c>
-      <c r="F14" s="82"/>
-      <c r="G14" s="82"/>
-      <c r="H14" s="82"/>
-      <c r="I14" s="82"/>
-      <c r="J14" s="82"/>
-      <c r="K14" s="82"/>
-      <c r="L14" s="82"/>
-      <c r="M14" s="82"/>
-      <c r="N14" s="82"/>
-      <c r="O14" s="83"/>
-      <c r="P14" s="14"/>
-      <c r="Q14" s="14"/>
-      <c r="R14" s="14"/>
-      <c r="S14" s="14"/>
+      <c r="F14" s="52"/>
+      <c r="G14" s="52"/>
+      <c r="H14" s="52"/>
+      <c r="I14" s="52"/>
+      <c r="J14" s="52"/>
+      <c r="K14" s="52"/>
+      <c r="L14" s="52"/>
+      <c r="M14" s="52"/>
+      <c r="N14" s="52"/>
+      <c r="O14" s="52"/>
+      <c r="P14" s="52"/>
+      <c r="Q14" s="52"/>
+      <c r="R14" s="52"/>
+      <c r="S14" s="53"/>
     </row>
     <row r="15" spans="2:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C15">
         <v>600</v>
       </c>
-      <c r="E15" s="72" t="s">
+      <c r="E15" s="92" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="66" t="s">
+      <c r="F15" s="88" t="s">
         <v>33</v>
       </c>
-      <c r="G15" s="66" t="s">
+      <c r="G15" s="88" t="s">
         <v>34</v>
       </c>
-      <c r="H15" s="66" t="s">
+      <c r="H15" s="88" t="s">
         <v>35</v>
       </c>
-      <c r="I15" s="66" t="s">
+      <c r="I15" s="88" t="s">
         <v>36</v>
       </c>
-      <c r="J15" s="66" t="s">
+      <c r="J15" s="88" t="s">
         <v>37</v>
       </c>
-      <c r="K15" s="66" t="s">
+      <c r="K15" s="99" t="s">
         <v>38</v>
       </c>
-      <c r="L15" s="66" t="s">
+      <c r="L15" s="101" t="s">
         <v>39</v>
       </c>
-      <c r="M15" s="66" t="s">
+      <c r="M15" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="N15" s="66" t="s">
+      <c r="N15" s="90" t="s">
         <v>41</v>
       </c>
-      <c r="O15" s="69" t="s">
+      <c r="O15" s="88" t="s">
         <v>42</v>
       </c>
+      <c r="P15" s="88" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q15" s="88" t="s">
+        <v>44</v>
+      </c>
+      <c r="R15" s="111" t="s">
+        <v>45</v>
+      </c>
+      <c r="S15" s="49" t="s">
+        <v>46</v>
+      </c>
+      <c r="U15" s="3"/>
+      <c r="V15" s="3"/>
+      <c r="W15" s="3"/>
     </row>
     <row r="16" spans="2:23" x14ac:dyDescent="0.25">
       <c r="C16">
         <v>650</v>
       </c>
-      <c r="E16" s="73"/>
-      <c r="F16" s="67"/>
-      <c r="G16" s="67"/>
-      <c r="H16" s="67"/>
-      <c r="I16" s="67"/>
-      <c r="J16" s="67"/>
-      <c r="K16" s="67"/>
-      <c r="L16" s="67" t="s">
-        <v>43</v>
-      </c>
-      <c r="M16" s="67"/>
-      <c r="N16" s="67"/>
-      <c r="O16" s="70"/>
+      <c r="E16" s="93"/>
+      <c r="F16" s="88"/>
+      <c r="G16" s="88"/>
+      <c r="H16" s="88"/>
+      <c r="I16" s="88"/>
+      <c r="J16" s="88"/>
+      <c r="K16" s="99"/>
+      <c r="L16" s="102"/>
+      <c r="M16" s="47"/>
+      <c r="N16" s="90"/>
+      <c r="O16" s="88" t="s">
+        <v>47</v>
+      </c>
+      <c r="P16" s="88"/>
+      <c r="Q16" s="88"/>
+      <c r="R16" s="112"/>
+      <c r="S16" s="49"/>
+      <c r="U16" s="3"/>
+      <c r="V16" s="3"/>
+      <c r="W16" s="3"/>
     </row>
-    <row r="17" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C17">
         <v>700</v>
       </c>
-      <c r="E17" s="74"/>
-      <c r="F17" s="68"/>
-      <c r="G17" s="68"/>
-      <c r="H17" s="68"/>
-      <c r="I17" s="68"/>
-      <c r="J17" s="68"/>
-      <c r="K17" s="68"/>
-      <c r="L17" s="68" t="s">
-        <v>44</v>
-      </c>
-      <c r="M17" s="68"/>
-      <c r="N17" s="68"/>
-      <c r="O17" s="71"/>
+      <c r="E17" s="94"/>
+      <c r="F17" s="89"/>
+      <c r="G17" s="89"/>
+      <c r="H17" s="89"/>
+      <c r="I17" s="89"/>
+      <c r="J17" s="89"/>
+      <c r="K17" s="100"/>
+      <c r="L17" s="103"/>
+      <c r="M17" s="48"/>
+      <c r="N17" s="91"/>
+      <c r="O17" s="89" t="s">
+        <v>48</v>
+      </c>
+      <c r="P17" s="89"/>
+      <c r="Q17" s="89"/>
+      <c r="R17" s="113"/>
+      <c r="S17" s="50"/>
+      <c r="U17" s="3"/>
+      <c r="V17" s="3"/>
+      <c r="W17" s="3"/>
     </row>
-    <row r="18" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="E18" s="15" t="s">
+    <row r="18" spans="3:23" x14ac:dyDescent="0.25">
+      <c r="E18" s="14" t="s">
         <v>20</v>
       </c>
       <c r="F18" s="6">
@@ -2248,137 +2677,209 @@
       <c r="J18" s="6">
         <v>6198</v>
       </c>
-      <c r="K18" s="6">
+      <c r="K18" s="28">
+        <v>48</v>
+      </c>
+      <c r="L18" s="36">
+        <f>J18*K18</f>
+        <v>297504</v>
+      </c>
+      <c r="M18" s="35">
+        <f>ROUND((L18-MIN($L$18:$L$22))/(MAX($L$18:$L$22)-MIN($L$18:$L$22)),2)</f>
+        <v>0.91</v>
+      </c>
+      <c r="N18" s="26">
         <v>827820</v>
       </c>
-      <c r="L18" s="6">
-        <f>ROUND((K18/G18),0)</f>
+      <c r="O18" s="6">
+        <f>ROUND((N18/G18),0)</f>
         <v>2123</v>
       </c>
-      <c r="M18" s="6">
-        <f>ROUND(1+4*(L18-MIN($L$18,$L$19,$L$20,$L$21,$L$22))/(MAX($L$18,$L$19,$L$20,$L$21,$L$22)-MIN($L$18,$L$19,$L$20,$L$21,$L$22)),0)</f>
+      <c r="P18" s="6">
+        <f>ROUND(1+4*(O18-MIN($O$18,$O$19,$O$20,$O$21,$O$22))/(MAX($O$18,$O$19,$O$20,$O$21,$O$22)-MIN($O$18,$O$19,$O$20,$O$21,$O$22)),0)</f>
         <v>2</v>
       </c>
-      <c r="N18" s="6">
+      <c r="Q18" s="6">
         <v>0.68513447400000005</v>
       </c>
-      <c r="O18" s="16">
+      <c r="R18" s="15">
         <v>30.747</v>
       </c>
+      <c r="S18" s="43">
+        <f>(P18*2)+(M18*1.5)</f>
+        <v>5.3650000000000002</v>
+      </c>
+      <c r="U18" s="3"/>
+      <c r="V18" s="3"/>
+      <c r="W18" s="3"/>
     </row>
-    <row r="19" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="E19" s="17" t="s">
+    <row r="19" spans="3:23" x14ac:dyDescent="0.25">
+      <c r="E19" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="F19" s="18">
+      <c r="F19" s="17">
         <v>24.181000000000001</v>
       </c>
-      <c r="G19" s="18">
+      <c r="G19" s="17">
         <v>1712</v>
       </c>
-      <c r="H19" s="18">
+      <c r="H19" s="17">
         <v>0.40799999999999997</v>
       </c>
-      <c r="I19" s="18">
+      <c r="I19" s="17">
         <v>14196</v>
       </c>
-      <c r="J19" s="18">
+      <c r="J19" s="17">
         <v>5792</v>
       </c>
-      <c r="K19" s="18">
+      <c r="K19" s="29">
+        <v>48</v>
+      </c>
+      <c r="L19" s="37">
+        <f t="shared" ref="L19:L22" si="13">J19*K19</f>
+        <v>278016</v>
+      </c>
+      <c r="M19" s="41">
+        <f t="shared" ref="M19:M22" si="14">ROUND((L19-MIN($L$18:$L$22))/(MAX($L$18:$L$22)-MIN($L$18:$L$22)),2)</f>
+        <v>0.84</v>
+      </c>
+      <c r="N19" s="32">
         <v>946080</v>
       </c>
-      <c r="L19" s="18">
-        <f>ROUND((K19/G19),0)</f>
+      <c r="O19" s="17">
+        <f>ROUND((N19/G19),0)</f>
         <v>553</v>
       </c>
-      <c r="M19" s="18">
-        <f>ROUND(1+4*(L19-MIN($L$18,$L$19,$L$20,$L$21,$L$22))/(MAX($L$18,$L$19,$L$20,$L$21,$L$22)-MIN($L$18,$L$19,$L$20,$L$21,$L$22)),0)</f>
+      <c r="P19" s="17">
+        <f>ROUND(1+4*(O19-MIN($O$18,$O$19,$O$20,$O$21,$O$22))/(MAX($O$18,$O$19,$O$20,$O$21,$O$22)-MIN($O$18,$O$19,$O$20,$O$21,$O$22)),0)</f>
         <v>1</v>
       </c>
-      <c r="N19" s="18">
+      <c r="Q19" s="17">
         <v>0.65204563999999998</v>
       </c>
-      <c r="O19" s="19">
+      <c r="R19" s="18">
         <v>120.622</v>
       </c>
+      <c r="S19" s="45">
+        <f t="shared" ref="S19:U22" si="15">(P19*2)+(M19*1.5)</f>
+        <v>3.26</v>
+      </c>
+      <c r="U19" s="3"/>
+      <c r="V19" s="3"/>
+      <c r="W19" s="3"/>
     </row>
-    <row r="20" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="E20" s="20" t="s">
+    <row r="20" spans="3:23" x14ac:dyDescent="0.25">
+      <c r="E20" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="F20" s="21">
+      <c r="F20" s="20">
         <v>21.507999999999999</v>
       </c>
-      <c r="G20" s="21">
+      <c r="G20" s="20">
         <v>183</v>
       </c>
-      <c r="H20" s="21">
+      <c r="H20" s="20">
         <v>0.45400000000000001</v>
       </c>
-      <c r="I20" s="21">
+      <c r="I20" s="20">
         <v>14788</v>
       </c>
-      <c r="J20" s="21">
+      <c r="J20" s="20">
         <v>6714</v>
       </c>
-      <c r="K20" s="21">
+      <c r="K20" s="30">
+        <v>48</v>
+      </c>
+      <c r="L20" s="38">
+        <f t="shared" si="13"/>
+        <v>322272</v>
+      </c>
+      <c r="M20" s="35">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="N20" s="33">
         <v>985500</v>
       </c>
-      <c r="L20" s="21">
-        <f>ROUND((K20/G20),0)</f>
+      <c r="O20" s="20">
+        <f>ROUND((N20/G20),0)</f>
         <v>5385</v>
       </c>
-      <c r="M20" s="21">
-        <f>ROUND(1+4*(L20-MIN($L$18,$L$19,$L$20,$L$21,$L$22))/(MAX($L$18,$L$19,$L$20,$L$21,$L$22)-MIN($L$18,$L$19,$L$20,$L$21,$L$22)),0)</f>
+      <c r="P20" s="20">
+        <f>ROUND(1+4*(O20-MIN($O$18,$O$19,$O$20,$O$21,$O$22))/(MAX($O$18,$O$19,$O$20,$O$21,$O$22)-MIN($O$18,$O$19,$O$20,$O$21,$O$22)),0)</f>
         <v>5</v>
       </c>
-      <c r="N20" s="21">
+      <c r="Q20" s="20">
         <v>0.84718826400000002</v>
       </c>
-      <c r="O20" s="22">
+      <c r="R20" s="21">
         <v>16.231000000000002</v>
       </c>
+      <c r="S20" s="43">
+        <f>(P20*2)+(M20*1.5)</f>
+        <v>11.5</v>
+      </c>
+      <c r="U20" s="3"/>
+      <c r="V20" s="3"/>
+      <c r="W20" s="3"/>
     </row>
-    <row r="21" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="E21" s="17" t="s">
+    <row r="21" spans="3:23" x14ac:dyDescent="0.25">
+      <c r="E21" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="F21" s="18">
+      <c r="F21" s="17">
         <v>16.437999999999999</v>
       </c>
-      <c r="G21" s="18">
+      <c r="G21" s="17">
         <v>249</v>
       </c>
-      <c r="H21" s="18">
+      <c r="H21" s="17">
         <v>0.40799999999999997</v>
       </c>
-      <c r="I21" s="18">
+      <c r="I21" s="17">
         <v>13013</v>
       </c>
-      <c r="J21" s="18">
+      <c r="J21" s="17">
         <v>5309</v>
       </c>
-      <c r="K21" s="18">
+      <c r="K21" s="29">
+        <v>48</v>
+      </c>
+      <c r="L21" s="39">
+        <f t="shared" si="13"/>
+        <v>254832</v>
+      </c>
+      <c r="M21" s="42">
+        <f t="shared" si="14"/>
+        <v>0.76</v>
+      </c>
+      <c r="N21" s="32">
         <v>867240</v>
       </c>
-      <c r="L21" s="18">
-        <f>ROUND((K21/G21),0)</f>
+      <c r="O21" s="17">
+        <f>ROUND((N21/G21),0)</f>
         <v>3483</v>
       </c>
-      <c r="M21" s="18">
-        <f>ROUND(1+4*(L21-MIN($L$18,$L$19,$L$20,$L$21,$L$22))/(MAX($L$18,$L$19,$L$20,$L$21,$L$22)-MIN($L$18,$L$19,$L$20,$L$21,$L$22)),0)</f>
+      <c r="P21" s="17">
+        <f>ROUND(1+4*(O21-MIN($O$18,$O$19,$O$20,$O$21,$O$22))/(MAX($O$18,$O$19,$O$20,$O$21,$O$22)-MIN($O$18,$O$19,$O$20,$O$21,$O$22)),0)</f>
         <v>3</v>
       </c>
-      <c r="N21" s="18">
+      <c r="Q21" s="17">
         <v>0.61268133700000005</v>
       </c>
-      <c r="O21" s="19">
+      <c r="R21" s="18">
         <v>21.013999999999999</v>
       </c>
+      <c r="S21" s="46">
+        <f t="shared" si="15"/>
+        <v>7.1400000000000006</v>
+      </c>
+      <c r="U21" s="3"/>
+      <c r="V21" s="3"/>
+      <c r="W21" s="3"/>
     </row>
-    <row r="22" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E22" s="23" t="s">
+    <row r="22" spans="3:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E22" s="22" t="s">
         <v>30</v>
       </c>
       <c r="F22" s="1">
@@ -2396,33 +2897,50 @@
       <c r="J22" s="1">
         <v>915</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="31">
+        <v>48</v>
+      </c>
+      <c r="L22" s="40">
+        <f t="shared" si="13"/>
+        <v>43920</v>
+      </c>
+      <c r="M22" s="34">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="N22" s="27">
         <v>670140</v>
       </c>
-      <c r="L22" s="1">
-        <f>ROUND((K22/G22),0)</f>
+      <c r="O22" s="1">
+        <f>ROUND((N22/G22),0)</f>
         <v>709</v>
       </c>
-      <c r="M22" s="1">
-        <f>ROUND(1+4*(L22-MIN($L$18,$L$19,$L$20,$L$21,$L$22))/(MAX($L$18,$L$19,$L$20,$L$21,$L$22)-MIN($L$18,$L$19,$L$20,$L$21,$L$22)),0)</f>
+      <c r="P22" s="1">
+        <f>ROUND(1+4*(O22-MIN($O$18,$O$19,$O$20,$O$21,$O$22))/(MAX($O$18,$O$19,$O$20,$O$21,$O$22)-MIN($O$18,$O$19,$O$20,$O$21,$O$22)),0)</f>
         <v>1</v>
       </c>
-      <c r="N22" s="1">
+      <c r="Q22" s="1">
         <v>0.13457212700000001</v>
       </c>
-      <c r="O22" s="24">
+      <c r="R22" s="23">
         <v>76.224000000000004</v>
       </c>
+      <c r="S22" s="44">
+        <f>(P22*2)+(M22*1.5)</f>
+        <v>2</v>
+      </c>
+      <c r="U22" s="3"/>
+      <c r="V22" s="3"/>
+      <c r="W22" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="108">
-    <mergeCell ref="E1:W1"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="K7:K8"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="I11:I12"/>
+  <mergeCells count="111">
+    <mergeCell ref="O3:O4"/>
+    <mergeCell ref="O15:O17"/>
+    <mergeCell ref="P15:P17"/>
+    <mergeCell ref="Q15:Q17"/>
+    <mergeCell ref="R15:R17"/>
+    <mergeCell ref="G15:G17"/>
     <mergeCell ref="F11:F12"/>
     <mergeCell ref="F9:F10"/>
     <mergeCell ref="F7:F8"/>
@@ -2432,16 +2950,6 @@
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="E9:E10"/>
     <mergeCell ref="E11:E12"/>
-    <mergeCell ref="O3:O4"/>
-    <mergeCell ref="L15:L17"/>
-    <mergeCell ref="M15:M17"/>
-    <mergeCell ref="N15:N17"/>
-    <mergeCell ref="O15:O17"/>
-    <mergeCell ref="G15:G17"/>
-    <mergeCell ref="H15:H17"/>
-    <mergeCell ref="I15:I17"/>
-    <mergeCell ref="J15:J17"/>
-    <mergeCell ref="K15:K17"/>
     <mergeCell ref="E15:E17"/>
     <mergeCell ref="F15:F17"/>
     <mergeCell ref="F3:F4"/>
@@ -2457,16 +2965,15 @@
     <mergeCell ref="L7:L8"/>
     <mergeCell ref="L5:L6"/>
     <mergeCell ref="L3:L4"/>
-    <mergeCell ref="E14:O14"/>
     <mergeCell ref="H3:H4"/>
     <mergeCell ref="H5:H6"/>
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="H9:H10"/>
     <mergeCell ref="H7:H8"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="K15:K17"/>
+    <mergeCell ref="L15:L17"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="K3:K4"/>
     <mergeCell ref="J3:J4"/>
     <mergeCell ref="N11:N12"/>
     <mergeCell ref="N9:N10"/>
@@ -2474,6 +2981,14 @@
     <mergeCell ref="I5:I6"/>
     <mergeCell ref="I7:I8"/>
     <mergeCell ref="I9:I10"/>
+    <mergeCell ref="H15:H17"/>
+    <mergeCell ref="I15:I17"/>
+    <mergeCell ref="J15:J17"/>
+    <mergeCell ref="N15:N17"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="I11:I12"/>
     <mergeCell ref="G11:G12"/>
     <mergeCell ref="K11:K12"/>
     <mergeCell ref="O11:O12"/>
@@ -2484,12 +2999,10 @@
     <mergeCell ref="M9:M10"/>
     <mergeCell ref="M7:M8"/>
     <mergeCell ref="M5:M6"/>
-    <mergeCell ref="Q3:Q4"/>
-    <mergeCell ref="R11:R12"/>
-    <mergeCell ref="R9:R10"/>
-    <mergeCell ref="R7:R8"/>
-    <mergeCell ref="R5:R6"/>
-    <mergeCell ref="R3:R4"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J5:J6"/>
     <mergeCell ref="P11:P12"/>
     <mergeCell ref="Q11:Q12"/>
     <mergeCell ref="Q9:Q10"/>
@@ -2499,16 +3012,19 @@
     <mergeCell ref="P5:P6"/>
     <mergeCell ref="P7:P8"/>
     <mergeCell ref="P9:P10"/>
-    <mergeCell ref="T11:T12"/>
-    <mergeCell ref="T9:T10"/>
-    <mergeCell ref="T7:T8"/>
-    <mergeCell ref="T5:T6"/>
-    <mergeCell ref="T3:T4"/>
-    <mergeCell ref="S11:S12"/>
     <mergeCell ref="S9:S10"/>
     <mergeCell ref="S7:S8"/>
     <mergeCell ref="S5:S6"/>
     <mergeCell ref="S3:S4"/>
+    <mergeCell ref="Q3:Q4"/>
+    <mergeCell ref="R11:R12"/>
+    <mergeCell ref="R9:R10"/>
+    <mergeCell ref="R7:R8"/>
+    <mergeCell ref="R5:R6"/>
+    <mergeCell ref="R3:R4"/>
+    <mergeCell ref="M15:M17"/>
+    <mergeCell ref="S15:S17"/>
+    <mergeCell ref="E14:S14"/>
     <mergeCell ref="W11:W12"/>
     <mergeCell ref="W9:W10"/>
     <mergeCell ref="W7:W8"/>
@@ -2524,6 +3040,12 @@
     <mergeCell ref="V5:V6"/>
     <mergeCell ref="V7:V8"/>
     <mergeCell ref="V9:V10"/>
+    <mergeCell ref="T11:T12"/>
+    <mergeCell ref="T9:T10"/>
+    <mergeCell ref="T7:T8"/>
+    <mergeCell ref="T5:T6"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="S11:S12"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H11 H9 H7 H3 H5" xr:uid="{27DD0D95-016E-4F9E-BAEF-71D55C9B5D21}">
@@ -2546,7 +3068,7 @@
   <sheetData>
     <row r="4" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>